<commit_message>
Update pilgrimage workbook data
</commit_message>
<xml_diff>
--- a/korean_catholic_holy_sites.xlsx
+++ b/korean_catholic_holy_sites.xlsx
@@ -8,14 +8,14 @@
     <sheet state="visible" name="추천코스" sheetId="3" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="2" name="_xlnm._FilterDatabase">'추천코스'!$A$1:$L$26</definedName>
+    <definedName hidden="1" localSheetId="2" name="_xlnm._FilterDatabase">'추천코스'!$A$1:$L$23</definedName>
   </definedNames>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1174" uniqueCount="616">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1273" uniqueCount="630">
   <si>
     <t>번호</t>
   </si>
@@ -587,7 +587,7 @@
     <t>62</t>
   </si>
   <si>
-    <t>묵호 순례 성당 (순교자 라 파트리치오 Patrick Reilly)</t>
+    <t>묵호 순례 성당</t>
   </si>
   <si>
     <t>강원특별자치도 동해시 발한로 161 (발한동)</t>
@@ -926,7 +926,7 @@
     <t>103</t>
   </si>
   <si>
-    <t>순교자 라 파트리치오(Patrick Reilly) 신부 순교터</t>
+    <t>순교자 라 파트리치오 신부 순교터</t>
   </si>
   <si>
     <t>강원특별자치도 강릉시 옥계면 낙풍리 산 16-2</t>
@@ -980,7 +980,7 @@
     <t>110</t>
   </si>
   <si>
-    <t>양양 성지 (순교자 이광재 디모테오)</t>
+    <t>양양 성지</t>
   </si>
   <si>
     <t>강원특별자치도 양양군 양양읍 군청길 17</t>
@@ -1715,138 +1715,120 @@
     <t>성지ID는 성지목록 시트의 성지명으로 생성된 ID와 연결됩니다.</t>
   </si>
   <si>
-    <t>naepo-pilgrimage</t>
-  </si>
-  <si>
-    <t>충남 내포 신앙의 길</t>
-  </si>
-  <si>
-    <t>충남 당진-서산</t>
-  </si>
-  <si>
-    <t>김대건 신부와 내포 교회</t>
+    <t>ganghwa_course</t>
+  </si>
+  <si>
+    <t>강화 순교 코스</t>
+  </si>
+  <si>
+    <t>인천-강화</t>
+  </si>
+  <si>
+    <t>강화도 내 순교성지</t>
+  </si>
+  <si>
+    <t>반나절</t>
+  </si>
+  <si>
+    <t>자동차</t>
+  </si>
+  <si>
+    <t xml:space="preserve">강화도 내 순례 코스입니다. </t>
+  </si>
+  <si>
+    <t>갑곶-순교-성지</t>
+  </si>
+  <si>
+    <t>진무영-순교-성지</t>
+  </si>
+  <si>
+    <t>north_gg_course</t>
+  </si>
+  <si>
+    <t>경기 북부-춘천지역 순례 코스</t>
+  </si>
+  <si>
+    <t>경기 북부-춘천</t>
+  </si>
+  <si>
+    <t>경기 북부-춘천 순교성지</t>
+  </si>
+  <si>
+    <t>2일</t>
+  </si>
+  <si>
+    <t xml:space="preserve">경기도 북부, 강원 춘천 순례 코스입니다. </t>
+  </si>
+  <si>
+    <t>참회와-속죄의-성당</t>
+  </si>
+  <si>
+    <t>신암리-성당</t>
+  </si>
+  <si>
+    <t>갈곡리-성당</t>
+  </si>
+  <si>
+    <t>양주-순교성지</t>
+  </si>
+  <si>
+    <t>성-남종삼-요한-·-순교자-남상교-아우구스티노-유택지</t>
+  </si>
+  <si>
+    <t>황사영-알렉시오-순교자-묘</t>
+  </si>
+  <si>
+    <t>포천-순교-성지-(복자-홍인-레오-순교터)</t>
+  </si>
+  <si>
+    <t>광암이벽요한세례자-진묘터와 생가터</t>
+  </si>
+  <si>
+    <t>소양로-순례-성당</t>
+  </si>
+  <si>
+    <t>죽림동-순교-성지</t>
+  </si>
+  <si>
+    <t>incheon_course</t>
+  </si>
+  <si>
+    <t>인천 순례코스</t>
+  </si>
+  <si>
+    <t>인천</t>
+  </si>
+  <si>
+    <t>인천 순교성지</t>
+  </si>
+  <si>
+    <t>대중교통</t>
+  </si>
+  <si>
+    <t xml:space="preserve">인천 순례 코스입니다. </t>
+  </si>
+  <si>
+    <t>이승훈-베드로-묘</t>
+  </si>
+  <si>
+    <t>제물진두-순교-성지</t>
+  </si>
+  <si>
+    <t>south_gg1_course</t>
+  </si>
+  <si>
+    <t>경기 남부 1 순례코스</t>
+  </si>
+  <si>
+    <t>경기남부</t>
+  </si>
+  <si>
+    <t>경기 남부 순교성지</t>
   </si>
   <si>
     <t>1일</t>
   </si>
   <si>
-    <t>자동차</t>
-  </si>
-  <si>
-    <t>솔뫼, 합덕, 신리, 해미를 잇는 대표 내포 순례 코스입니다.</t>
-  </si>
-  <si>
-    <t>사용여부가 Y인 행만 서비스에 표시하는 구조로 만들 예정입니다.</t>
-  </si>
-  <si>
-    <t>ganghwa_course</t>
-  </si>
-  <si>
-    <t>강화 순교 코스</t>
-  </si>
-  <si>
-    <t>인천-강화</t>
-  </si>
-  <si>
-    <t>강화도 내 순교성지</t>
-  </si>
-  <si>
-    <t>반나절</t>
-  </si>
-  <si>
-    <t xml:space="preserve">강화도 내 순례 코스입니다. </t>
-  </si>
-  <si>
-    <t>갑곶-순교-성지</t>
-  </si>
-  <si>
-    <t>진무영-순교-성지</t>
-  </si>
-  <si>
-    <t>north_gg_course</t>
-  </si>
-  <si>
-    <t>경기 북부-춘천지역 순례 코스</t>
-  </si>
-  <si>
-    <t>경기 북부-춘천</t>
-  </si>
-  <si>
-    <t>경기 북부-춘천 순교성지</t>
-  </si>
-  <si>
-    <t>2일</t>
-  </si>
-  <si>
-    <t xml:space="preserve">경기도 북부, 강원 춘천 순례 코스입니다. </t>
-  </si>
-  <si>
-    <t>참회와-속죄의-성당</t>
-  </si>
-  <si>
-    <t>신암리-성당</t>
-  </si>
-  <si>
-    <t>갈곡리-성당</t>
-  </si>
-  <si>
-    <t>양주-순교성지</t>
-  </si>
-  <si>
-    <t>성-남종삼-요한-·-순교자-남상교-아우구스티노-유택지</t>
-  </si>
-  <si>
-    <t>황사영-알렉시오-순교자-묘</t>
-  </si>
-  <si>
-    <t>포천-순교-성지-(복자-홍인-레오-순교터)</t>
-  </si>
-  <si>
-    <t>광암이벽요한세례자-진묘터와 생가터</t>
-  </si>
-  <si>
-    <t>소양로-순례-성당</t>
-  </si>
-  <si>
-    <t>죽림동-순교-성지</t>
-  </si>
-  <si>
-    <t>incheon_course</t>
-  </si>
-  <si>
-    <t>인천 순례코스</t>
-  </si>
-  <si>
-    <t>인천</t>
-  </si>
-  <si>
-    <t>인천 순교성지</t>
-  </si>
-  <si>
-    <t>대중교통</t>
-  </si>
-  <si>
-    <t xml:space="preserve">인천 순례 코스입니다. </t>
-  </si>
-  <si>
-    <t>이승훈-베드로-묘</t>
-  </si>
-  <si>
-    <t>제물진두-순교-성지</t>
-  </si>
-  <si>
-    <t>south_gg1_course</t>
-  </si>
-  <si>
-    <t>경기 남부 1 순례코스</t>
-  </si>
-  <si>
-    <t>경기남부</t>
-  </si>
-  <si>
-    <t>경기 남부 순교성지</t>
-  </si>
-  <si>
     <t xml:space="preserve">경기도 남부 안양, 수원, 화성 순례 코스입니다. </t>
   </si>
   <si>
@@ -1863,6 +1845,66 @@
   </si>
   <si>
     <t>남한산성-순교성지</t>
+  </si>
+  <si>
+    <t>south_gg3_course</t>
+  </si>
+  <si>
+    <t>경기 남부 3 순례코스</t>
+  </si>
+  <si>
+    <t xml:space="preserve">경기도 남부 용인, 이천, 안성 순례 코스입니다. </t>
+  </si>
+  <si>
+    <t>west_gw_course</t>
+  </si>
+  <si>
+    <t>강원, 충북 순례코스</t>
+  </si>
+  <si>
+    <t>강원서부,충북</t>
+  </si>
+  <si>
+    <t>강원 서부, 충북 순교성지</t>
+  </si>
+  <si>
+    <t xml:space="preserve">강원도 서부 횡성, 원주, 충북제천 순례코스입니다. </t>
+  </si>
+  <si>
+    <t>풍수원-성당</t>
+  </si>
+  <si>
+    <t>강원-감영</t>
+  </si>
+  <si>
+    <t>배론-성지</t>
+  </si>
+  <si>
+    <t>east_gw_course</t>
+  </si>
+  <si>
+    <t>강원 순례코스</t>
+  </si>
+  <si>
+    <t>강원동부</t>
+  </si>
+  <si>
+    <t>강원 순교성지</t>
+  </si>
+  <si>
+    <t xml:space="preserve">강원도 동부 양양, 삼척, 동해, 삼척 순례코스입니다. </t>
+  </si>
+  <si>
+    <t>양양-성지</t>
+  </si>
+  <si>
+    <t>순교자-라-파트리치오-신부-순교터</t>
+  </si>
+  <si>
+    <t>묵호-순례-성당</t>
+  </si>
+  <si>
+    <t>성내동-성당</t>
   </si>
 </sst>
 </file>
@@ -3143,7 +3185,7 @@
       <c r="C57" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="D57" s="1" t="s">
+      <c r="D57" s="2" t="s">
         <v>190</v>
       </c>
       <c r="E57" s="1" t="s">
@@ -3789,7 +3831,7 @@
       <c r="C95" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="D95" s="1" t="s">
+      <c r="D95" s="2" t="s">
         <v>303</v>
       </c>
       <c r="E95" s="1" t="s">
@@ -3891,7 +3933,7 @@
       <c r="C101" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="D101" s="1" t="s">
+      <c r="D101" s="2" t="s">
         <v>321</v>
       </c>
       <c r="E101" s="1" t="s">
@@ -7122,146 +7164,140 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="2" t="s">
         <v>566</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="2" t="s">
         <v>567</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="2" t="s">
         <v>568</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="2" t="s">
         <v>569</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="2" t="s">
         <v>570</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="F5" s="2" t="s">
         <v>571</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="G5" s="2" t="s">
         <v>572</v>
       </c>
-      <c r="H5" s="5">
+      <c r="H5" s="2">
         <v>1.0</v>
       </c>
-      <c r="I5" s="5" t="s">
-        <v>285</v>
-      </c>
-      <c r="J5" s="5" t="s">
-        <v>285</v>
+      <c r="I5" s="2" t="s">
+        <v>573</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="K5" s="5" t="s">
         <v>558</v>
       </c>
-      <c r="L5" s="5"/>
-      <c r="N5" s="1" t="s">
-        <v>573</v>
-      </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="2" t="s">
         <v>566</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="2" t="s">
         <v>567</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="2" t="s">
         <v>568</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="2" t="s">
         <v>569</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="2" t="s">
         <v>570</v>
       </c>
-      <c r="F6" s="5" t="s">
+      <c r="F6" s="2" t="s">
         <v>571</v>
       </c>
-      <c r="G6" s="5" t="s">
+      <c r="G6" s="2" t="s">
         <v>572</v>
       </c>
-      <c r="H6" s="5">
+      <c r="H6" s="2">
         <v>2.0</v>
       </c>
-      <c r="I6" s="5" t="s">
-        <v>488</v>
-      </c>
-      <c r="J6" s="5" t="s">
-        <v>488</v>
+      <c r="I6" s="2" t="s">
+        <v>574</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>443</v>
       </c>
       <c r="K6" s="5" t="s">
         <v>558</v>
       </c>
-      <c r="L6" s="5"/>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="s">
-        <v>566</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>567</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>568</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>569</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>570</v>
+      <c r="A7" s="2" t="s">
+        <v>575</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>576</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>577</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>578</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>579</v>
       </c>
       <c r="F7" s="5" t="s">
         <v>571</v>
       </c>
-      <c r="G7" s="5" t="s">
-        <v>572</v>
-      </c>
-      <c r="H7" s="5">
-        <v>3.0</v>
-      </c>
-      <c r="I7" s="5" t="s">
-        <v>312</v>
-      </c>
-      <c r="J7" s="5" t="s">
-        <v>312</v>
+      <c r="G7" s="2" t="s">
+        <v>580</v>
+      </c>
+      <c r="H7" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>581</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>452</v>
       </c>
       <c r="K7" s="5" t="s">
         <v>558</v>
       </c>
-      <c r="L7" s="5"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>577</v>
-      </c>
-      <c r="E8" s="2" t="s">
         <v>578</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="E8" s="6" t="s">
+        <v>579</v>
+      </c>
+      <c r="F8" s="5" t="s">
         <v>571</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="H8" s="2">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>37</v>
+        <v>315</v>
       </c>
       <c r="K8" s="5" t="s">
         <v>558</v>
@@ -7269,34 +7305,34 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>577</v>
-      </c>
-      <c r="E9" s="2" t="s">
         <v>578</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="E9" s="6" t="s">
+        <v>579</v>
+      </c>
+      <c r="F9" s="5" t="s">
         <v>571</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="H9" s="2">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>443</v>
+        <v>24</v>
       </c>
       <c r="K9" s="5" t="s">
         <v>558</v>
@@ -7304,34 +7340,34 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>582</v>
+        <v>575</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>583</v>
+        <v>576</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>584</v>
+        <v>577</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>585</v>
+        <v>578</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>586</v>
+        <v>579</v>
       </c>
       <c r="F10" s="5" t="s">
         <v>571</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>587</v>
+        <v>580</v>
       </c>
       <c r="H10" s="2">
-        <v>1.0</v>
+        <v>4.0</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>588</v>
+        <v>584</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>452</v>
+        <v>324</v>
       </c>
       <c r="K10" s="5" t="s">
         <v>558</v>
@@ -7339,34 +7375,34 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>582</v>
+        <v>575</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>583</v>
+        <v>576</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>584</v>
+        <v>577</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>585</v>
+        <v>578</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>586</v>
+        <v>579</v>
       </c>
       <c r="F11" s="5" t="s">
         <v>571</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>587</v>
+        <v>580</v>
       </c>
       <c r="H11" s="2">
-        <v>2.0</v>
+        <v>5.0</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>589</v>
+        <v>585</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>315</v>
+        <v>187</v>
       </c>
       <c r="K11" s="5" t="s">
         <v>558</v>
@@ -7374,34 +7410,34 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>582</v>
+        <v>575</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>583</v>
+        <v>576</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>584</v>
+        <v>577</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>585</v>
+        <v>578</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>586</v>
+        <v>579</v>
       </c>
       <c r="F12" s="5" t="s">
         <v>571</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>587</v>
+        <v>580</v>
       </c>
       <c r="H12" s="2">
-        <v>3.0</v>
+        <v>6.0</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>590</v>
+        <v>586</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>24</v>
+        <v>518</v>
       </c>
       <c r="K12" s="5" t="s">
         <v>558</v>
@@ -7409,34 +7445,34 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>582</v>
+        <v>575</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>583</v>
+        <v>576</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>584</v>
+        <v>577</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>585</v>
+        <v>578</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>586</v>
+        <v>579</v>
       </c>
       <c r="F13" s="5" t="s">
         <v>571</v>
       </c>
       <c r="G13" s="2" t="s">
+        <v>580</v>
+      </c>
+      <c r="H13" s="2">
+        <v>7.0</v>
+      </c>
+      <c r="I13" s="2" t="s">
         <v>587</v>
       </c>
-      <c r="H13" s="2">
-        <v>4.0</v>
-      </c>
-      <c r="I13" s="2" t="s">
-        <v>591</v>
-      </c>
       <c r="J13" s="1" t="s">
-        <v>324</v>
+        <v>473</v>
       </c>
       <c r="K13" s="5" t="s">
         <v>558</v>
@@ -7444,34 +7480,34 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>582</v>
+        <v>575</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>583</v>
+        <v>576</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>584</v>
+        <v>577</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>585</v>
+        <v>578</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>586</v>
+        <v>579</v>
       </c>
       <c r="F14" s="5" t="s">
         <v>571</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>587</v>
+        <v>580</v>
       </c>
       <c r="H14" s="2">
-        <v>5.0</v>
+        <v>8.0</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>592</v>
-      </c>
-      <c r="J14" s="1" t="s">
-        <v>187</v>
+        <v>588</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>509</v>
       </c>
       <c r="K14" s="5" t="s">
         <v>558</v>
@@ -7479,34 +7515,34 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>582</v>
+        <v>575</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>583</v>
+        <v>576</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>584</v>
+        <v>577</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>585</v>
+        <v>578</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>586</v>
+        <v>579</v>
       </c>
       <c r="F15" s="5" t="s">
         <v>571</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>587</v>
+        <v>580</v>
       </c>
       <c r="H15" s="2">
-        <v>6.0</v>
+        <v>9.0</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>593</v>
-      </c>
-      <c r="J15" s="1" t="s">
-        <v>518</v>
+        <v>589</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>279</v>
       </c>
       <c r="K15" s="5" t="s">
         <v>558</v>
@@ -7514,34 +7550,34 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>582</v>
+        <v>575</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>583</v>
+        <v>576</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>584</v>
+        <v>577</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>585</v>
+        <v>578</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>586</v>
+        <v>579</v>
       </c>
       <c r="F16" s="5" t="s">
         <v>571</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>587</v>
+        <v>580</v>
       </c>
       <c r="H16" s="2">
-        <v>7.0</v>
+        <v>10.0</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>594</v>
-      </c>
-      <c r="J16" s="1" t="s">
-        <v>473</v>
+        <v>590</v>
+      </c>
+      <c r="J16" s="2" t="s">
+        <v>428</v>
       </c>
       <c r="K16" s="5" t="s">
         <v>558</v>
@@ -7549,139 +7585,139 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>582</v>
+        <v>591</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>583</v>
+        <v>592</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>584</v>
+        <v>593</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>585</v>
-      </c>
-      <c r="E17" s="6" t="s">
-        <v>586</v>
-      </c>
-      <c r="F17" s="5" t="s">
-        <v>571</v>
+        <v>594</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>570</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>595</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>587</v>
+        <v>596</v>
       </c>
       <c r="H17" s="2">
-        <v>8.0</v>
+        <v>1.0</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>509</v>
+        <v>383</v>
       </c>
       <c r="K17" s="5" t="s">
         <v>558</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="2" t="s">
-        <v>582</v>
+        <v>591</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>583</v>
+        <v>592</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>584</v>
+        <v>593</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>585</v>
-      </c>
-      <c r="E18" s="6" t="s">
-        <v>586</v>
-      </c>
-      <c r="F18" s="5" t="s">
-        <v>571</v>
+        <v>594</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>570</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>595</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>587</v>
+        <v>596</v>
       </c>
       <c r="H18" s="2">
-        <v>9.0</v>
+        <v>2.0</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>596</v>
-      </c>
-      <c r="J18" s="2" t="s">
-        <v>279</v>
+        <v>598</v>
+      </c>
+      <c r="J18" s="1" t="s">
+        <v>410</v>
       </c>
       <c r="K18" s="5" t="s">
         <v>558</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" ht="15.75" customHeight="1">
       <c r="A19" s="2" t="s">
-        <v>582</v>
+        <v>599</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>583</v>
+        <v>600</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>584</v>
+        <v>601</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>585</v>
-      </c>
-      <c r="E19" s="6" t="s">
-        <v>586</v>
-      </c>
-      <c r="F19" s="5" t="s">
+        <v>602</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>603</v>
+      </c>
+      <c r="F19" s="2" t="s">
         <v>571</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>587</v>
+        <v>604</v>
       </c>
       <c r="H19" s="2">
-        <v>10.0</v>
-      </c>
-      <c r="I19" s="2" t="s">
-        <v>597</v>
-      </c>
-      <c r="J19" s="2" t="s">
-        <v>428</v>
+        <v>1.0</v>
+      </c>
+      <c r="I19" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="J19" s="1" t="s">
+        <v>288</v>
       </c>
       <c r="K19" s="5" t="s">
         <v>558</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="2" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>578</v>
+        <v>603</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>602</v>
+        <v>571</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="H20" s="2">
-        <v>1.0</v>
-      </c>
-      <c r="I20" s="2" t="s">
-        <v>604</v>
-      </c>
-      <c r="J20" s="2" t="s">
-        <v>383</v>
+        <v>2.0</v>
+      </c>
+      <c r="I20" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="J20" s="1" t="s">
+        <v>282</v>
       </c>
       <c r="K20" s="5" t="s">
         <v>558</v>
@@ -7689,34 +7725,34 @@
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="2" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>578</v>
+        <v>603</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>602</v>
+        <v>571</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="H21" s="2">
-        <v>2.0</v>
-      </c>
-      <c r="I21" s="2" t="s">
-        <v>605</v>
+        <v>3.0</v>
+      </c>
+      <c r="I21" s="1" t="s">
+        <v>297</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>410</v>
+        <v>297</v>
       </c>
       <c r="K21" s="5" t="s">
         <v>558</v>
@@ -7724,34 +7760,34 @@
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="2" t="s">
-        <v>606</v>
+        <v>599</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>607</v>
+        <v>600</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>608</v>
+        <v>601</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>609</v>
+        <v>602</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>570</v>
+        <v>603</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>571</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>610</v>
+        <v>604</v>
       </c>
       <c r="H22" s="2">
-        <v>1.0</v>
+        <v>4.0</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>288</v>
+        <v>132</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>288</v>
+        <v>132</v>
       </c>
       <c r="K22" s="5" t="s">
         <v>558</v>
@@ -7759,34 +7795,34 @@
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="2" t="s">
-        <v>606</v>
+        <v>599</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>607</v>
+        <v>600</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>608</v>
+        <v>601</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>609</v>
+        <v>602</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>570</v>
+        <v>603</v>
       </c>
       <c r="F23" s="2" t="s">
         <v>571</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>610</v>
+        <v>604</v>
       </c>
       <c r="H23" s="2">
-        <v>2.0</v>
+        <v>5.0</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>282</v>
+        <v>351</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>282</v>
+        <v>351</v>
       </c>
       <c r="K23" s="5" t="s">
         <v>558</v>
@@ -7794,34 +7830,34 @@
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="2" t="s">
+        <v>605</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>606</v>
       </c>
-      <c r="B24" s="2" t="s">
-        <v>607</v>
-      </c>
       <c r="C24" s="2" t="s">
-        <v>608</v>
+        <v>601</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>609</v>
+        <v>602</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>570</v>
+        <v>603</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>571</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>610</v>
+        <v>607</v>
       </c>
       <c r="H24" s="2">
-        <v>3.0</v>
-      </c>
-      <c r="I24" s="1" t="s">
-        <v>297</v>
-      </c>
-      <c r="J24" s="1" t="s">
-        <v>297</v>
+        <v>1.0</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="J24" s="2" t="s">
+        <v>98</v>
       </c>
       <c r="K24" s="5" t="s">
         <v>558</v>
@@ -7829,34 +7865,34 @@
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="2" t="s">
+        <v>605</v>
+      </c>
+      <c r="B25" s="2" t="s">
         <v>606</v>
       </c>
-      <c r="B25" s="2" t="s">
-        <v>607</v>
-      </c>
       <c r="C25" s="2" t="s">
-        <v>608</v>
+        <v>601</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>609</v>
+        <v>602</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>570</v>
+        <v>603</v>
       </c>
       <c r="F25" s="2" t="s">
         <v>571</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>610</v>
+        <v>607</v>
       </c>
       <c r="H25" s="2">
-        <v>4.0</v>
-      </c>
-      <c r="I25" s="1" t="s">
-        <v>132</v>
+        <v>2.0</v>
+      </c>
+      <c r="I25" s="2" t="s">
+        <v>608</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>132</v>
+        <v>175</v>
       </c>
       <c r="K25" s="5" t="s">
         <v>558</v>
@@ -7864,34 +7900,34 @@
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="2" t="s">
+        <v>605</v>
+      </c>
+      <c r="B26" s="2" t="s">
         <v>606</v>
       </c>
-      <c r="B26" s="2" t="s">
-        <v>607</v>
-      </c>
       <c r="C26" s="2" t="s">
-        <v>608</v>
+        <v>601</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>609</v>
+        <v>602</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>570</v>
+        <v>603</v>
       </c>
       <c r="F26" s="2" t="s">
         <v>571</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>610</v>
+        <v>607</v>
       </c>
       <c r="H26" s="2">
-        <v>5.0</v>
+        <v>3.0</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>351</v>
+        <v>318</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>351</v>
+        <v>318</v>
       </c>
       <c r="K26" s="5" t="s">
         <v>558</v>
@@ -7899,34 +7935,34 @@
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="2" t="s">
-        <v>611</v>
+        <v>605</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>612</v>
+        <v>606</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>608</v>
+        <v>601</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>609</v>
+        <v>602</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>570</v>
+        <v>603</v>
       </c>
       <c r="F27" s="2" t="s">
         <v>571</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>613</v>
+        <v>607</v>
       </c>
       <c r="H27" s="2">
-        <v>1.0</v>
-      </c>
-      <c r="I27" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="J27" s="2" t="s">
-        <v>98</v>
+        <v>4.0</v>
+      </c>
+      <c r="I27" s="1" t="s">
+        <v>455</v>
+      </c>
+      <c r="J27" s="1" t="s">
+        <v>455</v>
       </c>
       <c r="K27" s="5" t="s">
         <v>558</v>
@@ -7934,34 +7970,34 @@
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="2" t="s">
-        <v>611</v>
+        <v>605</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>612</v>
+        <v>606</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>608</v>
+        <v>601</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>609</v>
+        <v>602</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>570</v>
+        <v>603</v>
       </c>
       <c r="F28" s="2" t="s">
         <v>571</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>613</v>
+        <v>607</v>
       </c>
       <c r="H28" s="2">
-        <v>2.0</v>
+        <v>5.0</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>614</v>
+        <v>609</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>175</v>
+        <v>135</v>
       </c>
       <c r="K28" s="5" t="s">
         <v>558</v>
@@ -7969,34 +8005,34 @@
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="2" t="s">
+        <v>610</v>
+      </c>
+      <c r="B29" s="2" t="s">
         <v>611</v>
       </c>
-      <c r="B29" s="2" t="s">
-        <v>612</v>
-      </c>
       <c r="C29" s="2" t="s">
-        <v>608</v>
+        <v>601</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>609</v>
+        <v>602</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>570</v>
+        <v>603</v>
       </c>
       <c r="F29" s="2" t="s">
         <v>571</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="H29" s="2">
-        <v>3.0</v>
+        <v>1.0</v>
       </c>
       <c r="I29" s="1" t="s">
-        <v>318</v>
+        <v>375</v>
       </c>
       <c r="J29" s="1" t="s">
-        <v>318</v>
+        <v>375</v>
       </c>
       <c r="K29" s="5" t="s">
         <v>558</v>
@@ -8004,34 +8040,34 @@
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="2" t="s">
+        <v>610</v>
+      </c>
+      <c r="B30" s="2" t="s">
         <v>611</v>
       </c>
-      <c r="B30" s="2" t="s">
-        <v>612</v>
-      </c>
       <c r="C30" s="2" t="s">
-        <v>608</v>
+        <v>601</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>609</v>
+        <v>602</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>570</v>
+        <v>603</v>
       </c>
       <c r="F30" s="2" t="s">
         <v>571</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="H30" s="2">
-        <v>4.0</v>
+        <v>2.0</v>
       </c>
       <c r="I30" s="1" t="s">
-        <v>455</v>
+        <v>148</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>455</v>
+        <v>148</v>
       </c>
       <c r="K30" s="5" t="s">
         <v>558</v>
@@ -8039,49 +8075,389 @@
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="2" t="s">
+        <v>610</v>
+      </c>
+      <c r="B31" s="2" t="s">
         <v>611</v>
       </c>
-      <c r="B31" s="2" t="s">
-        <v>612</v>
-      </c>
       <c r="C31" s="2" t="s">
-        <v>608</v>
+        <v>601</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>609</v>
+        <v>602</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>570</v>
+        <v>603</v>
       </c>
       <c r="F31" s="2" t="s">
         <v>571</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="H31" s="2">
-        <v>5.0</v>
-      </c>
-      <c r="I31" s="2" t="s">
-        <v>615</v>
+        <v>3.0</v>
+      </c>
+      <c r="I31" s="1" t="s">
+        <v>327</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>135</v>
+        <v>327</v>
       </c>
       <c r="K31" s="5" t="s">
         <v>558</v>
       </c>
     </row>
-    <row r="32" ht="15.75" customHeight="1"/>
-    <row r="33" ht="15.75" customHeight="1"/>
-    <row r="34" ht="15.75" customHeight="1"/>
-    <row r="35" ht="15.75" customHeight="1"/>
-    <row r="36" ht="15.75" customHeight="1"/>
-    <row r="37" ht="15.75" customHeight="1"/>
-    <row r="38" ht="15.75" customHeight="1"/>
-    <row r="39" ht="15.75" customHeight="1"/>
-    <row r="40" ht="15.75" customHeight="1"/>
-    <row r="41" ht="15.75" customHeight="1"/>
+    <row r="32" ht="15.75" customHeight="1">
+      <c r="A32" s="2" t="s">
+        <v>610</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>611</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>601</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>602</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>603</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>612</v>
+      </c>
+      <c r="H32" s="2">
+        <v>4.0</v>
+      </c>
+      <c r="I32" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="J32" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="K32" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="33" ht="15.75" customHeight="1">
+      <c r="A33" s="2" t="s">
+        <v>610</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>611</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>601</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>602</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>603</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>612</v>
+      </c>
+      <c r="H33" s="2">
+        <v>5.0</v>
+      </c>
+      <c r="I33" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="J33" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="K33" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="34" ht="15.75" customHeight="1">
+      <c r="A34" s="2" t="s">
+        <v>613</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>614</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>615</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>616</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>603</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>617</v>
+      </c>
+      <c r="H34" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="I34" s="2" t="s">
+        <v>618</v>
+      </c>
+      <c r="J34" s="1" t="s">
+        <v>476</v>
+      </c>
+      <c r="K34" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="35" ht="15.75" customHeight="1">
+      <c r="A35" s="2" t="s">
+        <v>613</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>614</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>615</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>616</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>603</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>617</v>
+      </c>
+      <c r="H35" s="2">
+        <v>2.0</v>
+      </c>
+      <c r="I35" s="2" t="s">
+        <v>619</v>
+      </c>
+      <c r="J35" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="K35" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="36" ht="15.75" customHeight="1">
+      <c r="A36" s="2" t="s">
+        <v>613</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>614</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>615</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>616</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>603</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>617</v>
+      </c>
+      <c r="H36" s="2">
+        <v>3.0</v>
+      </c>
+      <c r="I36" s="2" t="s">
+        <v>585</v>
+      </c>
+      <c r="J36" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="K36" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="37" ht="15.75" customHeight="1">
+      <c r="A37" s="2" t="s">
+        <v>613</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>614</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>615</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>616</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>603</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>617</v>
+      </c>
+      <c r="H37" s="2">
+        <v>4.0</v>
+      </c>
+      <c r="I37" s="2" t="s">
+        <v>620</v>
+      </c>
+      <c r="J37" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="K37" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="38" ht="15.75" customHeight="1">
+      <c r="A38" s="2" t="s">
+        <v>621</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>622</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>623</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>624</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>603</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>625</v>
+      </c>
+      <c r="H38" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="I38" s="2" t="s">
+        <v>626</v>
+      </c>
+      <c r="J38" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="K38" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="39" ht="15.75" customHeight="1">
+      <c r="A39" s="2" t="s">
+        <v>621</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>622</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>623</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>624</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>603</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>625</v>
+      </c>
+      <c r="H39" s="2">
+        <v>2.0</v>
+      </c>
+      <c r="I39" s="2" t="s">
+        <v>627</v>
+      </c>
+      <c r="J39" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="K39" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="40" ht="15.75" customHeight="1">
+      <c r="A40" s="2" t="s">
+        <v>621</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>622</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>623</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>624</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>603</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>625</v>
+      </c>
+      <c r="H40" s="2">
+        <v>3.0</v>
+      </c>
+      <c r="I40" s="2" t="s">
+        <v>628</v>
+      </c>
+      <c r="J40" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="K40" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="41" ht="15.75" customHeight="1">
+      <c r="A41" s="2" t="s">
+        <v>621</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>622</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>623</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>624</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>603</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>625</v>
+      </c>
+      <c r="H41" s="2">
+        <v>4.0</v>
+      </c>
+      <c r="I41" s="2" t="s">
+        <v>629</v>
+      </c>
+      <c r="J41" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="K41" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
     <row r="42" ht="15.75" customHeight="1"/>
     <row r="43" ht="15.75" customHeight="1"/>
     <row r="44" ht="15.75" customHeight="1"/>
@@ -9038,11 +9414,8 @@
     <row r="995" ht="15.75" customHeight="1"/>
     <row r="996" ht="15.75" customHeight="1"/>
     <row r="997" ht="15.75" customHeight="1"/>
-    <row r="998" ht="15.75" customHeight="1"/>
-    <row r="999" ht="15.75" customHeight="1"/>
-    <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="$A$1:$L$26"/>
+  <autoFilter ref="$A$1:$L$23"/>
   <printOptions/>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
   <pageSetup orientation="landscape"/>

</xml_diff>

<commit_message>
Update pilgrimage workbook content
</commit_message>
<xml_diff>
--- a/korean_catholic_holy_sites.xlsx
+++ b/korean_catholic_holy_sites.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1483" uniqueCount="650">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1883" uniqueCount="707">
   <si>
     <t>번호</t>
   </si>
@@ -488,7 +488,7 @@
     <t>48</t>
   </si>
   <si>
-    <t>대산성당 구한선 타대오 성지(교구 순교복자 묘소)</t>
+    <t>대산성당</t>
   </si>
   <si>
     <t>경상남도 함안군 대산면 대산중앙로 183</t>
@@ -1097,7 +1097,7 @@
     <t>127</t>
   </si>
   <si>
-    <t>용수 성지 (성 김대건 신부 표착기념관)</t>
+    <t>용수 성지</t>
   </si>
   <si>
     <t>제주특별자치도 제주시 한경면 용수1길 108</t>
@@ -1400,7 +1400,7 @@
     <t>164</t>
   </si>
   <si>
-    <t>청주 읍성 순교 성지</t>
+    <t>서운동 순교 성지</t>
   </si>
   <si>
     <t>충청북도 청주시 상당구 대성로 41 서운동 성당</t>
@@ -1745,7 +1745,7 @@
     <t>north_gg_course</t>
   </si>
   <si>
-    <t>경기 북부-춘천지역 순례 코스</t>
+    <t>경기 평화의 순례</t>
   </si>
   <si>
     <t>경기 북부-춘천</t>
@@ -1817,7 +1817,7 @@
     <t>south_gg1_course</t>
   </si>
   <si>
-    <t>경기 남부 1 순례코스</t>
+    <t>경기 기억과 믿음의 길</t>
   </si>
   <si>
     <t>경기남부</t>
@@ -1835,7 +1835,7 @@
     <t>south_gg2_course</t>
   </si>
   <si>
-    <t>경기 남부 2 순례코스</t>
+    <t>경기 은총의 길</t>
   </si>
   <si>
     <t xml:space="preserve">경기도 남부 하남, 광주, 양평 순례 코스입니다. </t>
@@ -1850,7 +1850,7 @@
     <t>south_gg3_course</t>
   </si>
   <si>
-    <t>경기 남부 3 순례코스</t>
+    <t>경기 빛을 따라 걷는 길</t>
   </si>
   <si>
     <t xml:space="preserve">경기도 남부 용인, 이천, 안성 순례 코스입니다. </t>
@@ -1928,7 +1928,7 @@
     <t>north_cn2_course</t>
   </si>
   <si>
-    <t>충남1 순례코스</t>
+    <t>충남 고요한 기도의 길</t>
   </si>
   <si>
     <t xml:space="preserve">충청남도 서산, 홍성 순례코스입니다 </t>
@@ -1937,7 +1937,7 @@
     <t>north_cn3_course</t>
   </si>
   <si>
-    <t>충남2 순례코스</t>
+    <t>충남 신앙의 발자취</t>
   </si>
   <si>
     <t xml:space="preserve">충청남도 보령, 청양, 공주 순례코스입니다 </t>
@@ -1949,7 +1949,7 @@
     <t>north_cn4_course</t>
   </si>
   <si>
-    <t>충남3 순례코스</t>
+    <t>충남 마음의 순례</t>
   </si>
   <si>
     <t xml:space="preserve">충청남도 부여, 서천 순례코스입니다 </t>
@@ -1965,6 +1965,177 @@
   </si>
   <si>
     <t>산막골성지-/-작은재성지</t>
+  </si>
+  <si>
+    <t>cj_course</t>
+  </si>
+  <si>
+    <t>청주 성지로 향하는 여정</t>
+  </si>
+  <si>
+    <t>충청북도</t>
+  </si>
+  <si>
+    <t>충청북도 순교성지</t>
+  </si>
+  <si>
+    <t xml:space="preserve">충청북도 진천, 청주, 보은 순례코스입니다 </t>
+  </si>
+  <si>
+    <t>배티-순교-성지</t>
+  </si>
+  <si>
+    <t>서운동-순교-성지</t>
+  </si>
+  <si>
+    <t>멍에목-성지</t>
+  </si>
+  <si>
+    <t>ad_course</t>
+  </si>
+  <si>
+    <t>문경 믿음의 발자취</t>
+  </si>
+  <si>
+    <t>경상북도</t>
+  </si>
+  <si>
+    <t>경상북도 순교성지</t>
+  </si>
+  <si>
+    <t xml:space="preserve">충청북도 괴산, 경상북도 문경 순례코스입니다 </t>
+  </si>
+  <si>
+    <t>연풍-순교-성지</t>
+  </si>
+  <si>
+    <t>마원-성지</t>
+  </si>
+  <si>
+    <t>진안리-성지</t>
+  </si>
+  <si>
+    <t>여우목-성지</t>
+  </si>
+  <si>
+    <t>north_jj_course</t>
+  </si>
+  <si>
+    <t>전북 순교자의 길</t>
+  </si>
+  <si>
+    <t>전라북도</t>
+  </si>
+  <si>
+    <t>전라북도 순교성지</t>
+  </si>
+  <si>
+    <t xml:space="preserve">전라북도 익산, 충청남도 금산 순례코스입니다 </t>
+  </si>
+  <si>
+    <t>여산-하늘의-문-성당</t>
+  </si>
+  <si>
+    <t>center_jj_course</t>
+  </si>
+  <si>
+    <t>전북 위로의 순례길</t>
+  </si>
+  <si>
+    <t xml:space="preserve">전라북도 김제, 전주 순례코스입니다 </t>
+  </si>
+  <si>
+    <t>gj_course</t>
+  </si>
+  <si>
+    <t>전라도 함께하는 순례길</t>
+  </si>
+  <si>
+    <t>전라남도</t>
+  </si>
+  <si>
+    <t>전라남도 순교성지</t>
+  </si>
+  <si>
+    <t xml:space="preserve">전라북도 고창, 전라남도 영광, 나주, 목포, 곡성 순례코스입니다. </t>
+  </si>
+  <si>
+    <t>고창-개갑-순교성지</t>
+  </si>
+  <si>
+    <t>나주-순교자-기념성당</t>
+  </si>
+  <si>
+    <t>곡성성당-옥터</t>
+  </si>
+  <si>
+    <t>dg_course</t>
+  </si>
+  <si>
+    <t>경상북도 신앙의 발자취</t>
+  </si>
+  <si>
+    <t xml:space="preserve">경상북도 대구, 경주 순례코스입니다. </t>
+  </si>
+  <si>
+    <t>신나무골-성지</t>
+  </si>
+  <si>
+    <t>경상-감영과-옥-터</t>
+  </si>
+  <si>
+    <t>진목정-성지</t>
+  </si>
+  <si>
+    <t>경주-관아와-옥-터</t>
+  </si>
+  <si>
+    <t>ms_course</t>
+  </si>
+  <si>
+    <t>경상남도 숲과 기도의 길</t>
+  </si>
+  <si>
+    <t>경상남도</t>
+  </si>
+  <si>
+    <t>경상남도 순교성지</t>
+  </si>
+  <si>
+    <t xml:space="preserve">경상남도 창원, 함안, 거제 순례코스입니다. </t>
+  </si>
+  <si>
+    <t>명례-성지</t>
+  </si>
+  <si>
+    <t>복자-박대식-빅토리노-묘</t>
+  </si>
+  <si>
+    <t>복자-정찬문-안토니오-묘소</t>
+  </si>
+  <si>
+    <t>복자-윤봉문-요셉-성지</t>
+  </si>
+  <si>
+    <t>jj_course</t>
+  </si>
+  <si>
+    <t>제주도 고요한 침묵</t>
+  </si>
+  <si>
+    <t>제주도</t>
+  </si>
+  <si>
+    <t>제주도 순교성지</t>
+  </si>
+  <si>
+    <t xml:space="preserve">제주도 순례코스입니다. </t>
+  </si>
+  <si>
+    <t>김기량-순교-기념관</t>
+  </si>
+  <si>
+    <t>용수-성지</t>
   </si>
 </sst>
 </file>
@@ -3059,7 +3230,7 @@
       <c r="C46" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D46" s="1" t="s">
+      <c r="D46" s="2" t="s">
         <v>157</v>
       </c>
       <c r="E46" s="1" t="s">
@@ -4215,7 +4386,7 @@
       <c r="C114" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="D114" s="1" t="s">
+      <c r="D114" s="2" t="s">
         <v>360</v>
       </c>
       <c r="E114" s="1" t="s">
@@ -4793,7 +4964,7 @@
       <c r="C148" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D148" s="1" t="s">
+      <c r="D148" s="2" t="s">
         <v>461</v>
       </c>
       <c r="E148" s="1" t="s">
@@ -9254,46 +9425,1406 @@
         <v>558</v>
       </c>
     </row>
-    <row r="63" ht="15.75" customHeight="1"/>
-    <row r="64" ht="15.75" customHeight="1"/>
-    <row r="65" ht="15.75" customHeight="1"/>
-    <row r="66" ht="15.75" customHeight="1"/>
-    <row r="67" ht="15.75" customHeight="1"/>
-    <row r="68" ht="15.75" customHeight="1"/>
-    <row r="69" ht="15.75" customHeight="1"/>
-    <row r="70" ht="15.75" customHeight="1"/>
-    <row r="71" ht="15.75" customHeight="1"/>
-    <row r="72" ht="15.75" customHeight="1"/>
-    <row r="73" ht="15.75" customHeight="1"/>
-    <row r="74" ht="15.75" customHeight="1"/>
-    <row r="75" ht="15.75" customHeight="1"/>
-    <row r="76" ht="15.75" customHeight="1"/>
-    <row r="77" ht="15.75" customHeight="1"/>
-    <row r="78" ht="15.75" customHeight="1"/>
-    <row r="79" ht="15.75" customHeight="1"/>
-    <row r="80" ht="15.75" customHeight="1"/>
-    <row r="81" ht="15.75" customHeight="1"/>
-    <row r="82" ht="15.75" customHeight="1"/>
-    <row r="83" ht="15.75" customHeight="1"/>
-    <row r="84" ht="15.75" customHeight="1"/>
-    <row r="85" ht="15.75" customHeight="1"/>
-    <row r="86" ht="15.75" customHeight="1"/>
-    <row r="87" ht="15.75" customHeight="1"/>
-    <row r="88" ht="15.75" customHeight="1"/>
-    <row r="89" ht="15.75" customHeight="1"/>
-    <row r="90" ht="15.75" customHeight="1"/>
-    <row r="91" ht="15.75" customHeight="1"/>
-    <row r="92" ht="15.75" customHeight="1"/>
-    <row r="93" ht="15.75" customHeight="1"/>
-    <row r="94" ht="15.75" customHeight="1"/>
-    <row r="95" ht="15.75" customHeight="1"/>
-    <row r="96" ht="15.75" customHeight="1"/>
-    <row r="97" ht="15.75" customHeight="1"/>
-    <row r="98" ht="15.75" customHeight="1"/>
-    <row r="99" ht="15.75" customHeight="1"/>
-    <row r="100" ht="15.75" customHeight="1"/>
-    <row r="101" ht="15.75" customHeight="1"/>
-    <row r="102" ht="15.75" customHeight="1"/>
+    <row r="63" ht="15.75" customHeight="1">
+      <c r="A63" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>651</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>652</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>653</v>
+      </c>
+      <c r="E63" s="2" t="s">
+        <v>603</v>
+      </c>
+      <c r="F63" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G63" s="2" t="s">
+        <v>654</v>
+      </c>
+      <c r="H63" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="I63" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="J63" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="K63" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="64" ht="15.75" customHeight="1">
+      <c r="A64" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>651</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>652</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>653</v>
+      </c>
+      <c r="E64" s="2" t="s">
+        <v>603</v>
+      </c>
+      <c r="F64" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G64" s="2" t="s">
+        <v>654</v>
+      </c>
+      <c r="H64" s="2">
+        <v>2.0</v>
+      </c>
+      <c r="I64" s="2" t="s">
+        <v>655</v>
+      </c>
+      <c r="J64" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="K64" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="65" ht="15.75" customHeight="1">
+      <c r="A65" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>651</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>652</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>653</v>
+      </c>
+      <c r="E65" s="2" t="s">
+        <v>603</v>
+      </c>
+      <c r="F65" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G65" s="2" t="s">
+        <v>654</v>
+      </c>
+      <c r="H65" s="2">
+        <v>3.0</v>
+      </c>
+      <c r="I65" s="2" t="s">
+        <v>656</v>
+      </c>
+      <c r="J65" s="2" t="s">
+        <v>461</v>
+      </c>
+      <c r="K65" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="66" ht="15.75" customHeight="1">
+      <c r="A66" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>651</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>652</v>
+      </c>
+      <c r="D66" s="2" t="s">
+        <v>653</v>
+      </c>
+      <c r="E66" s="2" t="s">
+        <v>603</v>
+      </c>
+      <c r="F66" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G66" s="2" t="s">
+        <v>654</v>
+      </c>
+      <c r="H66" s="2">
+        <v>4.0</v>
+      </c>
+      <c r="I66" s="2" t="s">
+        <v>657</v>
+      </c>
+      <c r="J66" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="K66" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="67" ht="15.75" customHeight="1">
+      <c r="A67" s="2" t="s">
+        <v>658</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>659</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>660</v>
+      </c>
+      <c r="D67" s="2" t="s">
+        <v>661</v>
+      </c>
+      <c r="E67" s="2" t="s">
+        <v>603</v>
+      </c>
+      <c r="F67" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G67" s="2" t="s">
+        <v>662</v>
+      </c>
+      <c r="H67" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="I67" s="2" t="s">
+        <v>663</v>
+      </c>
+      <c r="J67" s="1" t="s">
+        <v>342</v>
+      </c>
+      <c r="K67" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="68" ht="15.75" customHeight="1">
+      <c r="A68" s="2" t="s">
+        <v>658</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>659</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>660</v>
+      </c>
+      <c r="D68" s="2" t="s">
+        <v>661</v>
+      </c>
+      <c r="E68" s="2" t="s">
+        <v>603</v>
+      </c>
+      <c r="F68" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G68" s="2" t="s">
+        <v>662</v>
+      </c>
+      <c r="H68" s="2">
+        <v>2.0</v>
+      </c>
+      <c r="I68" s="2" t="s">
+        <v>664</v>
+      </c>
+      <c r="J68" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="K68" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="69" ht="15.75" customHeight="1">
+      <c r="A69" s="2" t="s">
+        <v>658</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>659</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>660</v>
+      </c>
+      <c r="D69" s="2" t="s">
+        <v>661</v>
+      </c>
+      <c r="E69" s="2" t="s">
+        <v>603</v>
+      </c>
+      <c r="F69" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G69" s="2" t="s">
+        <v>662</v>
+      </c>
+      <c r="H69" s="2">
+        <v>3.0</v>
+      </c>
+      <c r="I69" s="2" t="s">
+        <v>665</v>
+      </c>
+      <c r="J69" s="1" t="s">
+        <v>449</v>
+      </c>
+      <c r="K69" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="70" ht="15.75" customHeight="1">
+      <c r="A70" s="2" t="s">
+        <v>658</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>659</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>660</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>661</v>
+      </c>
+      <c r="E70" s="2" t="s">
+        <v>603</v>
+      </c>
+      <c r="F70" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G70" s="2" t="s">
+        <v>662</v>
+      </c>
+      <c r="H70" s="2">
+        <v>4.0</v>
+      </c>
+      <c r="I70" s="2" t="s">
+        <v>666</v>
+      </c>
+      <c r="J70" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="K70" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="71" ht="15.75" customHeight="1">
+      <c r="A71" s="2" t="s">
+        <v>667</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>668</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>669</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>670</v>
+      </c>
+      <c r="E71" s="2" t="s">
+        <v>603</v>
+      </c>
+      <c r="F71" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G71" s="2" t="s">
+        <v>671</v>
+      </c>
+      <c r="H71" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="I71" s="1" t="s">
+        <v>446</v>
+      </c>
+      <c r="J71" s="1" t="s">
+        <v>446</v>
+      </c>
+      <c r="K71" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="72" ht="15.75" customHeight="1">
+      <c r="A72" s="2" t="s">
+        <v>667</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>668</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>669</v>
+      </c>
+      <c r="D72" s="2" t="s">
+        <v>670</v>
+      </c>
+      <c r="E72" s="2" t="s">
+        <v>603</v>
+      </c>
+      <c r="F72" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G72" s="2" t="s">
+        <v>671</v>
+      </c>
+      <c r="H72" s="2">
+        <v>2.0</v>
+      </c>
+      <c r="I72" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="J72" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="K72" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="73" ht="15.75" customHeight="1">
+      <c r="A73" s="2" t="s">
+        <v>667</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>668</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>669</v>
+      </c>
+      <c r="D73" s="2" t="s">
+        <v>670</v>
+      </c>
+      <c r="E73" s="2" t="s">
+        <v>603</v>
+      </c>
+      <c r="F73" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G73" s="2" t="s">
+        <v>671</v>
+      </c>
+      <c r="H73" s="2">
+        <v>3.0</v>
+      </c>
+      <c r="I73" s="2" t="s">
+        <v>672</v>
+      </c>
+      <c r="J73" s="1" t="s">
+        <v>336</v>
+      </c>
+      <c r="K73" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="74" ht="15.75" customHeight="1">
+      <c r="A74" s="2" t="s">
+        <v>667</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>668</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>669</v>
+      </c>
+      <c r="D74" s="2" t="s">
+        <v>670</v>
+      </c>
+      <c r="E74" s="2" t="s">
+        <v>603</v>
+      </c>
+      <c r="F74" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G74" s="2" t="s">
+        <v>671</v>
+      </c>
+      <c r="H74" s="2">
+        <v>4.0</v>
+      </c>
+      <c r="I74" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="J74" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="K74" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="75" ht="15.75" customHeight="1">
+      <c r="A75" s="2" t="s">
+        <v>673</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>674</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>669</v>
+      </c>
+      <c r="D75" s="2" t="s">
+        <v>670</v>
+      </c>
+      <c r="E75" s="2" t="s">
+        <v>603</v>
+      </c>
+      <c r="F75" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G75" s="2" t="s">
+        <v>675</v>
+      </c>
+      <c r="H75" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="I75" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="J75" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="K75" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="76" ht="15.75" customHeight="1">
+      <c r="A76" s="2" t="s">
+        <v>673</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>674</v>
+      </c>
+      <c r="C76" s="2" t="s">
+        <v>669</v>
+      </c>
+      <c r="D76" s="2" t="s">
+        <v>670</v>
+      </c>
+      <c r="E76" s="2" t="s">
+        <v>603</v>
+      </c>
+      <c r="F76" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G76" s="2" t="s">
+        <v>675</v>
+      </c>
+      <c r="H76" s="2">
+        <v>2.0</v>
+      </c>
+      <c r="I76" s="1" t="s">
+        <v>464</v>
+      </c>
+      <c r="J76" s="1" t="s">
+        <v>464</v>
+      </c>
+      <c r="K76" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="77" ht="15.75" customHeight="1">
+      <c r="A77" s="2" t="s">
+        <v>673</v>
+      </c>
+      <c r="B77" s="2" t="s">
+        <v>674</v>
+      </c>
+      <c r="C77" s="2" t="s">
+        <v>669</v>
+      </c>
+      <c r="D77" s="2" t="s">
+        <v>670</v>
+      </c>
+      <c r="E77" s="2" t="s">
+        <v>603</v>
+      </c>
+      <c r="F77" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G77" s="2" t="s">
+        <v>675</v>
+      </c>
+      <c r="H77" s="2">
+        <v>3.0</v>
+      </c>
+      <c r="I77" s="1" t="s">
+        <v>401</v>
+      </c>
+      <c r="J77" s="1" t="s">
+        <v>401</v>
+      </c>
+      <c r="K77" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="78" ht="15.75" customHeight="1">
+      <c r="A78" s="2" t="s">
+        <v>673</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>674</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>669</v>
+      </c>
+      <c r="D78" s="2" t="s">
+        <v>670</v>
+      </c>
+      <c r="E78" s="2" t="s">
+        <v>603</v>
+      </c>
+      <c r="F78" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G78" s="2" t="s">
+        <v>675</v>
+      </c>
+      <c r="H78" s="2">
+        <v>4.0</v>
+      </c>
+      <c r="I78" s="1" t="s">
+        <v>404</v>
+      </c>
+      <c r="J78" s="1" t="s">
+        <v>404</v>
+      </c>
+      <c r="K78" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="79" ht="15.75" customHeight="1">
+      <c r="A79" s="2" t="s">
+        <v>673</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>674</v>
+      </c>
+      <c r="C79" s="2" t="s">
+        <v>669</v>
+      </c>
+      <c r="D79" s="2" t="s">
+        <v>670</v>
+      </c>
+      <c r="E79" s="2" t="s">
+        <v>603</v>
+      </c>
+      <c r="F79" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G79" s="2" t="s">
+        <v>675</v>
+      </c>
+      <c r="H79" s="2">
+        <v>5.0</v>
+      </c>
+      <c r="I79" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="J79" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="K79" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="80" ht="15.75" customHeight="1">
+      <c r="A80" s="2" t="s">
+        <v>673</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>674</v>
+      </c>
+      <c r="C80" s="2" t="s">
+        <v>669</v>
+      </c>
+      <c r="D80" s="2" t="s">
+        <v>670</v>
+      </c>
+      <c r="E80" s="2" t="s">
+        <v>603</v>
+      </c>
+      <c r="F80" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G80" s="2" t="s">
+        <v>675</v>
+      </c>
+      <c r="H80" s="2">
+        <v>6.0</v>
+      </c>
+      <c r="I80" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="J80" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="K80" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="81" ht="15.75" customHeight="1">
+      <c r="A81" s="2" t="s">
+        <v>673</v>
+      </c>
+      <c r="B81" s="2" t="s">
+        <v>674</v>
+      </c>
+      <c r="C81" s="2" t="s">
+        <v>669</v>
+      </c>
+      <c r="D81" s="2" t="s">
+        <v>670</v>
+      </c>
+      <c r="E81" s="2" t="s">
+        <v>603</v>
+      </c>
+      <c r="F81" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G81" s="2" t="s">
+        <v>675</v>
+      </c>
+      <c r="H81" s="2">
+        <v>7.0</v>
+      </c>
+      <c r="I81" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="J81" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="K81" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="82" ht="15.75" customHeight="1">
+      <c r="A82" s="2" t="s">
+        <v>673</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>674</v>
+      </c>
+      <c r="C82" s="2" t="s">
+        <v>669</v>
+      </c>
+      <c r="D82" s="2" t="s">
+        <v>670</v>
+      </c>
+      <c r="E82" s="2" t="s">
+        <v>603</v>
+      </c>
+      <c r="F82" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G82" s="2" t="s">
+        <v>675</v>
+      </c>
+      <c r="H82" s="2">
+        <v>8.0</v>
+      </c>
+      <c r="I82" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="J82" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="K82" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="83" ht="15.75" customHeight="1">
+      <c r="A83" s="2" t="s">
+        <v>676</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>677</v>
+      </c>
+      <c r="C83" s="2" t="s">
+        <v>678</v>
+      </c>
+      <c r="D83" s="2" t="s">
+        <v>679</v>
+      </c>
+      <c r="E83" s="2" t="s">
+        <v>579</v>
+      </c>
+      <c r="F83" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G83" s="2" t="s">
+        <v>680</v>
+      </c>
+      <c r="H83" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="I83" s="2" t="s">
+        <v>681</v>
+      </c>
+      <c r="J83" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="K83" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="84" ht="15.75" customHeight="1">
+      <c r="A84" s="2" t="s">
+        <v>676</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>677</v>
+      </c>
+      <c r="C84" s="2" t="s">
+        <v>678</v>
+      </c>
+      <c r="D84" s="2" t="s">
+        <v>679</v>
+      </c>
+      <c r="E84" s="2" t="s">
+        <v>579</v>
+      </c>
+      <c r="F84" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G84" s="2" t="s">
+        <v>680</v>
+      </c>
+      <c r="H84" s="2">
+        <v>2.0</v>
+      </c>
+      <c r="I84" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="J84" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="K84" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="85" ht="15.75" customHeight="1">
+      <c r="A85" s="2" t="s">
+        <v>676</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>677</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>678</v>
+      </c>
+      <c r="D85" s="2" t="s">
+        <v>679</v>
+      </c>
+      <c r="E85" s="2" t="s">
+        <v>579</v>
+      </c>
+      <c r="F85" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G85" s="2" t="s">
+        <v>680</v>
+      </c>
+      <c r="H85" s="2">
+        <v>3.0</v>
+      </c>
+      <c r="I85" s="2" t="s">
+        <v>682</v>
+      </c>
+      <c r="J85" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="K85" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="86" ht="15.75" customHeight="1">
+      <c r="A86" s="2" t="s">
+        <v>676</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>677</v>
+      </c>
+      <c r="C86" s="2" t="s">
+        <v>678</v>
+      </c>
+      <c r="D86" s="2" t="s">
+        <v>679</v>
+      </c>
+      <c r="E86" s="2" t="s">
+        <v>579</v>
+      </c>
+      <c r="F86" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G86" s="2" t="s">
+        <v>680</v>
+      </c>
+      <c r="H86" s="2">
+        <v>4.0</v>
+      </c>
+      <c r="I86" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="J86" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="K86" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="87" ht="15.75" customHeight="1">
+      <c r="A87" s="2" t="s">
+        <v>676</v>
+      </c>
+      <c r="B87" s="2" t="s">
+        <v>677</v>
+      </c>
+      <c r="C87" s="2" t="s">
+        <v>678</v>
+      </c>
+      <c r="D87" s="2" t="s">
+        <v>679</v>
+      </c>
+      <c r="E87" s="2" t="s">
+        <v>579</v>
+      </c>
+      <c r="F87" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G87" s="2" t="s">
+        <v>680</v>
+      </c>
+      <c r="H87" s="2">
+        <v>5.0</v>
+      </c>
+      <c r="I87" s="2" t="s">
+        <v>683</v>
+      </c>
+      <c r="J87" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="K87" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="88" ht="15.75" customHeight="1">
+      <c r="A88" s="2" t="s">
+        <v>684</v>
+      </c>
+      <c r="B88" s="2" t="s">
+        <v>685</v>
+      </c>
+      <c r="C88" s="2" t="s">
+        <v>660</v>
+      </c>
+      <c r="D88" s="2" t="s">
+        <v>661</v>
+      </c>
+      <c r="E88" s="2" t="s">
+        <v>579</v>
+      </c>
+      <c r="F88" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G88" s="2" t="s">
+        <v>686</v>
+      </c>
+      <c r="H88" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="I88" s="1" t="s">
+        <v>485</v>
+      </c>
+      <c r="J88" s="1" t="s">
+        <v>485</v>
+      </c>
+      <c r="K88" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="89" ht="15.75" customHeight="1">
+      <c r="A89" s="2" t="s">
+        <v>684</v>
+      </c>
+      <c r="B89" s="2" t="s">
+        <v>685</v>
+      </c>
+      <c r="C89" s="2" t="s">
+        <v>660</v>
+      </c>
+      <c r="D89" s="2" t="s">
+        <v>661</v>
+      </c>
+      <c r="E89" s="2" t="s">
+        <v>579</v>
+      </c>
+      <c r="F89" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G89" s="2" t="s">
+        <v>686</v>
+      </c>
+      <c r="H89" s="2">
+        <v>2.0</v>
+      </c>
+      <c r="I89" s="2" t="s">
+        <v>687</v>
+      </c>
+      <c r="J89" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="K89" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="90" ht="15.75" customHeight="1">
+      <c r="A90" s="2" t="s">
+        <v>684</v>
+      </c>
+      <c r="B90" s="2" t="s">
+        <v>685</v>
+      </c>
+      <c r="C90" s="2" t="s">
+        <v>660</v>
+      </c>
+      <c r="D90" s="2" t="s">
+        <v>661</v>
+      </c>
+      <c r="E90" s="2" t="s">
+        <v>579</v>
+      </c>
+      <c r="F90" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G90" s="2" t="s">
+        <v>686</v>
+      </c>
+      <c r="H90" s="2">
+        <v>3.0</v>
+      </c>
+      <c r="I90" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="J90" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="K90" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="91" ht="15.75" customHeight="1">
+      <c r="A91" s="2" t="s">
+        <v>684</v>
+      </c>
+      <c r="B91" s="2" t="s">
+        <v>685</v>
+      </c>
+      <c r="C91" s="2" t="s">
+        <v>660</v>
+      </c>
+      <c r="D91" s="2" t="s">
+        <v>661</v>
+      </c>
+      <c r="E91" s="2" t="s">
+        <v>579</v>
+      </c>
+      <c r="F91" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G91" s="2" t="s">
+        <v>686</v>
+      </c>
+      <c r="H91" s="2">
+        <v>4.0</v>
+      </c>
+      <c r="I91" s="2" t="s">
+        <v>688</v>
+      </c>
+      <c r="J91" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="K91" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="92" ht="15.75" customHeight="1">
+      <c r="A92" s="2" t="s">
+        <v>684</v>
+      </c>
+      <c r="B92" s="2" t="s">
+        <v>685</v>
+      </c>
+      <c r="C92" s="2" t="s">
+        <v>660</v>
+      </c>
+      <c r="D92" s="2" t="s">
+        <v>661</v>
+      </c>
+      <c r="E92" s="2" t="s">
+        <v>579</v>
+      </c>
+      <c r="F92" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G92" s="2" t="s">
+        <v>686</v>
+      </c>
+      <c r="H92" s="2">
+        <v>5.0</v>
+      </c>
+      <c r="I92" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="J92" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="K92" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="93" ht="15.75" customHeight="1">
+      <c r="A93" s="2" t="s">
+        <v>684</v>
+      </c>
+      <c r="B93" s="2" t="s">
+        <v>685</v>
+      </c>
+      <c r="C93" s="2" t="s">
+        <v>660</v>
+      </c>
+      <c r="D93" s="2" t="s">
+        <v>661</v>
+      </c>
+      <c r="E93" s="2" t="s">
+        <v>579</v>
+      </c>
+      <c r="F93" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G93" s="2" t="s">
+        <v>686</v>
+      </c>
+      <c r="H93" s="2">
+        <v>6.0</v>
+      </c>
+      <c r="I93" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="J93" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="K93" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="94" ht="15.75" customHeight="1">
+      <c r="A94" s="2" t="s">
+        <v>684</v>
+      </c>
+      <c r="B94" s="2" t="s">
+        <v>685</v>
+      </c>
+      <c r="C94" s="2" t="s">
+        <v>660</v>
+      </c>
+      <c r="D94" s="2" t="s">
+        <v>661</v>
+      </c>
+      <c r="E94" s="2" t="s">
+        <v>579</v>
+      </c>
+      <c r="F94" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G94" s="2" t="s">
+        <v>686</v>
+      </c>
+      <c r="H94" s="2">
+        <v>7.0</v>
+      </c>
+      <c r="I94" s="2" t="s">
+        <v>689</v>
+      </c>
+      <c r="J94" s="1" t="s">
+        <v>440</v>
+      </c>
+      <c r="K94" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="95" ht="15.75" customHeight="1">
+      <c r="A95" s="2" t="s">
+        <v>684</v>
+      </c>
+      <c r="B95" s="2" t="s">
+        <v>685</v>
+      </c>
+      <c r="C95" s="2" t="s">
+        <v>660</v>
+      </c>
+      <c r="D95" s="2" t="s">
+        <v>661</v>
+      </c>
+      <c r="E95" s="2" t="s">
+        <v>579</v>
+      </c>
+      <c r="F95" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G95" s="2" t="s">
+        <v>686</v>
+      </c>
+      <c r="H95" s="2">
+        <v>8.0</v>
+      </c>
+      <c r="I95" s="2" t="s">
+        <v>690</v>
+      </c>
+      <c r="J95" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="K95" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="96" ht="15.75" customHeight="1">
+      <c r="A96" s="2" t="s">
+        <v>691</v>
+      </c>
+      <c r="B96" s="2" t="s">
+        <v>692</v>
+      </c>
+      <c r="C96" s="2" t="s">
+        <v>693</v>
+      </c>
+      <c r="D96" s="2" t="s">
+        <v>694</v>
+      </c>
+      <c r="E96" s="2" t="s">
+        <v>579</v>
+      </c>
+      <c r="F96" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G96" s="2" t="s">
+        <v>695</v>
+      </c>
+      <c r="H96" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="I96" s="2" t="s">
+        <v>696</v>
+      </c>
+      <c r="J96" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="K96" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="97" ht="15.75" customHeight="1">
+      <c r="A97" s="2" t="s">
+        <v>691</v>
+      </c>
+      <c r="B97" s="2" t="s">
+        <v>692</v>
+      </c>
+      <c r="C97" s="2" t="s">
+        <v>693</v>
+      </c>
+      <c r="D97" s="2" t="s">
+        <v>694</v>
+      </c>
+      <c r="E97" s="2" t="s">
+        <v>579</v>
+      </c>
+      <c r="F97" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G97" s="2" t="s">
+        <v>695</v>
+      </c>
+      <c r="H97" s="2">
+        <v>2.0</v>
+      </c>
+      <c r="I97" s="2" t="s">
+        <v>697</v>
+      </c>
+      <c r="J97" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="K97" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="98" ht="15.75" customHeight="1">
+      <c r="A98" s="2" t="s">
+        <v>691</v>
+      </c>
+      <c r="B98" s="2" t="s">
+        <v>692</v>
+      </c>
+      <c r="C98" s="2" t="s">
+        <v>693</v>
+      </c>
+      <c r="D98" s="2" t="s">
+        <v>694</v>
+      </c>
+      <c r="E98" s="2" t="s">
+        <v>579</v>
+      </c>
+      <c r="F98" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G98" s="2" t="s">
+        <v>695</v>
+      </c>
+      <c r="H98" s="2">
+        <v>3.0</v>
+      </c>
+      <c r="I98" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="J98" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="K98" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="99" ht="15.75" customHeight="1">
+      <c r="A99" s="2" t="s">
+        <v>691</v>
+      </c>
+      <c r="B99" s="2" t="s">
+        <v>692</v>
+      </c>
+      <c r="C99" s="2" t="s">
+        <v>693</v>
+      </c>
+      <c r="D99" s="2" t="s">
+        <v>694</v>
+      </c>
+      <c r="E99" s="2" t="s">
+        <v>579</v>
+      </c>
+      <c r="F99" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G99" s="2" t="s">
+        <v>695</v>
+      </c>
+      <c r="H99" s="2">
+        <v>4.0</v>
+      </c>
+      <c r="I99" s="2" t="s">
+        <v>698</v>
+      </c>
+      <c r="J99" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K99" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="100" ht="15.75" customHeight="1">
+      <c r="A100" s="2" t="s">
+        <v>691</v>
+      </c>
+      <c r="B100" s="2" t="s">
+        <v>692</v>
+      </c>
+      <c r="C100" s="2" t="s">
+        <v>693</v>
+      </c>
+      <c r="D100" s="2" t="s">
+        <v>694</v>
+      </c>
+      <c r="E100" s="2" t="s">
+        <v>579</v>
+      </c>
+      <c r="F100" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G100" s="2" t="s">
+        <v>695</v>
+      </c>
+      <c r="H100" s="2">
+        <v>5.0</v>
+      </c>
+      <c r="I100" s="2" t="s">
+        <v>699</v>
+      </c>
+      <c r="J100" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="K100" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="101" ht="15.75" customHeight="1">
+      <c r="A101" s="2" t="s">
+        <v>700</v>
+      </c>
+      <c r="B101" s="2" t="s">
+        <v>701</v>
+      </c>
+      <c r="C101" s="2" t="s">
+        <v>702</v>
+      </c>
+      <c r="D101" s="2" t="s">
+        <v>703</v>
+      </c>
+      <c r="E101" s="2" t="s">
+        <v>570</v>
+      </c>
+      <c r="F101" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G101" s="2" t="s">
+        <v>704</v>
+      </c>
+      <c r="H101" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="I101" s="2" t="s">
+        <v>705</v>
+      </c>
+      <c r="J101" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="K101" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="102" ht="15.75" customHeight="1">
+      <c r="A102" s="2" t="s">
+        <v>700</v>
+      </c>
+      <c r="B102" s="2" t="s">
+        <v>701</v>
+      </c>
+      <c r="C102" s="2" t="s">
+        <v>702</v>
+      </c>
+      <c r="D102" s="2" t="s">
+        <v>703</v>
+      </c>
+      <c r="E102" s="2" t="s">
+        <v>570</v>
+      </c>
+      <c r="F102" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G102" s="2" t="s">
+        <v>704</v>
+      </c>
+      <c r="H102" s="2">
+        <v>2.0</v>
+      </c>
+      <c r="I102" s="2" t="s">
+        <v>706</v>
+      </c>
+      <c r="J102" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="K102" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
     <row r="103" ht="15.75" customHeight="1"/>
     <row r="104" ht="15.75" customHeight="1"/>
     <row r="105" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
Update pilgrimage workbook IDs
</commit_message>
<xml_diff>
--- a/korean_catholic_holy_sites.xlsx
+++ b/korean_catholic_holy_sites.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2010" uniqueCount="714">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2010" uniqueCount="716">
   <si>
     <t>번호</t>
   </si>
@@ -1799,16 +1799,16 @@
     <t>양주-순교성지</t>
   </si>
   <si>
+    <t>황사영-알렉시오-순교자-묘</t>
+  </si>
+  <si>
     <t>성-남종삼-요한과-가족-순교자-묘소</t>
   </si>
   <si>
-    <t>황사영-알렉시오-순교자-묘</t>
-  </si>
-  <si>
-    <t>포천-순교-성지-(복자-홍인-레오-순교터)</t>
-  </si>
-  <si>
-    <t>광암이벽요한세례자-진묘터와 생가터</t>
+    <t>포천-순교-성지-복자-홍인-레오-순교터</t>
+  </si>
+  <si>
+    <t>광암이벽요한세례자-진묘터와-생가터</t>
   </si>
   <si>
     <t>소양로-순례-성당</t>
@@ -1877,6 +1877,9 @@
     <t xml:space="preserve">경기도 남부 용인, 이천, 안성 순례 코스입니다. </t>
   </si>
   <si>
+    <t>은이골배마실성지</t>
+  </si>
+  <si>
     <t>west_gw_course</t>
   </si>
   <si>
@@ -1898,7 +1901,7 @@
     <t>강원-감영</t>
   </si>
   <si>
-    <t>성-남종삼-요한-·-순교자-남상교-아우구스티노-유택지</t>
+    <t>성-남종삼-요한--순교자-남상교-아우구스티노-유택지</t>
   </si>
   <si>
     <t>배론-성지</t>
@@ -1985,7 +1988,7 @@
     <t>서짓골-성지</t>
   </si>
   <si>
-    <t>산막골성지-/-작은재성지</t>
+    <t>산막골성지--작은재성지</t>
   </si>
   <si>
     <t>cj_course</t>
@@ -2100,6 +2103,9 @@
   </si>
   <si>
     <t>신나무골-성지</t>
+  </si>
+  <si>
+    <t>비산날뫼성당</t>
   </si>
   <si>
     <t>경상-감영과-옥-터</t>
@@ -8098,7 +8104,7 @@
         <v>594</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>253</v>
+        <v>518</v>
       </c>
       <c r="K24" s="5" t="s">
         <v>557</v>
@@ -8133,7 +8139,7 @@
         <v>595</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>518</v>
+        <v>253</v>
       </c>
       <c r="K25" s="5" t="s">
         <v>557</v>
@@ -8724,8 +8730,8 @@
       <c r="H42" s="2">
         <v>1.0</v>
       </c>
-      <c r="I42" s="1" t="s">
-        <v>375</v>
+      <c r="I42" s="2" t="s">
+        <v>620</v>
       </c>
       <c r="J42" s="1" t="s">
         <v>375</v>
@@ -8876,16 +8882,16 @@
     </row>
     <row r="47" ht="15.75" customHeight="1">
       <c r="A47" s="2" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="E47" s="2" t="s">
         <v>570</v>
@@ -8894,13 +8900,13 @@
         <v>580</v>
       </c>
       <c r="G47" s="2" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="H47" s="2">
         <v>1.0</v>
       </c>
       <c r="I47" s="2" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="J47" s="1" t="s">
         <v>476</v>
@@ -8911,16 +8917,16 @@
     </row>
     <row r="48" ht="15.75" customHeight="1">
       <c r="A48" s="2" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="E48" s="2" t="s">
         <v>570</v>
@@ -8929,13 +8935,13 @@
         <v>580</v>
       </c>
       <c r="G48" s="2" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="H48" s="2">
         <v>2.0</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="J48" s="1" t="s">
         <v>49</v>
@@ -8946,16 +8952,16 @@
     </row>
     <row r="49" ht="15.75" customHeight="1">
       <c r="A49" s="2" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="E49" s="2" t="s">
         <v>570</v>
@@ -8964,13 +8970,13 @@
         <v>580</v>
       </c>
       <c r="G49" s="2" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="H49" s="2">
         <v>3.0</v>
       </c>
       <c r="I49" s="2" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="J49" s="1" t="s">
         <v>187</v>
@@ -8981,16 +8987,16 @@
     </row>
     <row r="50" ht="15.75" customHeight="1">
       <c r="A50" s="2" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="E50" s="2" t="s">
         <v>570</v>
@@ -8999,13 +9005,13 @@
         <v>580</v>
       </c>
       <c r="G50" s="2" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="H50" s="2">
         <v>4.0</v>
       </c>
       <c r="I50" s="2" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="J50" s="1" t="s">
         <v>271</v>
@@ -9016,16 +9022,16 @@
     </row>
     <row r="51" ht="15.75" customHeight="1">
       <c r="A51" s="2" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="E51" s="2" t="s">
         <v>570</v>
@@ -9034,13 +9040,13 @@
         <v>580</v>
       </c>
       <c r="G51" s="2" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="H51" s="2">
         <v>1.0</v>
       </c>
       <c r="I51" s="2" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="J51" s="2" t="s">
         <v>321</v>
@@ -9051,16 +9057,16 @@
     </row>
     <row r="52" ht="15.75" customHeight="1">
       <c r="A52" s="2" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="E52" s="2" t="s">
         <v>570</v>
@@ -9069,13 +9075,13 @@
         <v>580</v>
       </c>
       <c r="G52" s="2" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="H52" s="2">
         <v>2.0</v>
       </c>
       <c r="I52" s="2" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="J52" s="2" t="s">
         <v>303</v>
@@ -9086,16 +9092,16 @@
     </row>
     <row r="53" ht="15.75" customHeight="1">
       <c r="A53" s="2" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="E53" s="2" t="s">
         <v>570</v>
@@ -9104,13 +9110,13 @@
         <v>580</v>
       </c>
       <c r="G53" s="2" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="H53" s="2">
         <v>3.0</v>
       </c>
       <c r="I53" s="2" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="J53" s="2" t="s">
         <v>190</v>
@@ -9121,16 +9127,16 @@
     </row>
     <row r="54" ht="15.75" customHeight="1">
       <c r="A54" s="2" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="E54" s="2" t="s">
         <v>570</v>
@@ -9139,13 +9145,13 @@
         <v>580</v>
       </c>
       <c r="G54" s="2" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="H54" s="2">
         <v>4.0</v>
       </c>
       <c r="I54" s="2" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="J54" s="1" t="s">
         <v>262</v>
@@ -9156,16 +9162,16 @@
     </row>
     <row r="55" ht="15.75" customHeight="1">
       <c r="A55" s="2" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E55" s="2" t="s">
         <v>570</v>
@@ -9174,7 +9180,7 @@
         <v>580</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="H55" s="2">
         <v>1.0</v>
@@ -9191,16 +9197,16 @@
     </row>
     <row r="56" ht="15.75" customHeight="1">
       <c r="A56" s="2" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E56" s="2" t="s">
         <v>570</v>
@@ -9209,7 +9215,7 @@
         <v>580</v>
       </c>
       <c r="G56" s="2" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="H56" s="2">
         <v>2.0</v>
@@ -9226,16 +9232,16 @@
     </row>
     <row r="57" ht="15.75" customHeight="1">
       <c r="A57" s="2" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E57" s="2" t="s">
         <v>570</v>
@@ -9244,7 +9250,7 @@
         <v>580</v>
       </c>
       <c r="G57" s="2" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="H57" s="2">
         <v>3.0</v>
@@ -9261,16 +9267,16 @@
     </row>
     <row r="58" ht="15.75" customHeight="1">
       <c r="A58" s="2" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E58" s="2" t="s">
         <v>570</v>
@@ -9279,7 +9285,7 @@
         <v>580</v>
       </c>
       <c r="G58" s="2" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="H58" s="2">
         <v>4.0</v>
@@ -9296,16 +9302,16 @@
     </row>
     <row r="59" ht="15.75" customHeight="1">
       <c r="A59" s="2" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E59" s="2" t="s">
         <v>570</v>
@@ -9314,7 +9320,7 @@
         <v>580</v>
       </c>
       <c r="G59" s="2" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="H59" s="2">
         <v>5.0</v>
@@ -9331,16 +9337,16 @@
     </row>
     <row r="60" ht="15.75" customHeight="1">
       <c r="A60" s="2" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E60" s="2" t="s">
         <v>570</v>
@@ -9349,7 +9355,7 @@
         <v>580</v>
       </c>
       <c r="G60" s="2" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="H60" s="2">
         <v>6.0</v>
@@ -9366,16 +9372,16 @@
     </row>
     <row r="61" ht="15.75" customHeight="1">
       <c r="A61" s="2" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E61" s="2" t="s">
         <v>570</v>
@@ -9384,7 +9390,7 @@
         <v>580</v>
       </c>
       <c r="G61" s="2" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="H61" s="2">
         <v>7.0</v>
@@ -9401,16 +9407,16 @@
     </row>
     <row r="62" ht="15.75" customHeight="1">
       <c r="A62" s="2" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E62" s="2" t="s">
         <v>570</v>
@@ -9419,7 +9425,7 @@
         <v>580</v>
       </c>
       <c r="G62" s="2" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="H62" s="2">
         <v>8.0</v>
@@ -9436,16 +9442,16 @@
     </row>
     <row r="63" ht="15.75" customHeight="1">
       <c r="A63" s="2" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E63" s="2" t="s">
         <v>570</v>
@@ -9454,7 +9460,7 @@
         <v>580</v>
       </c>
       <c r="G63" s="2" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="H63" s="2">
         <v>1.0</v>
@@ -9471,16 +9477,16 @@
     </row>
     <row r="64" ht="15.75" customHeight="1">
       <c r="A64" s="2" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E64" s="2" t="s">
         <v>570</v>
@@ -9489,7 +9495,7 @@
         <v>580</v>
       </c>
       <c r="G64" s="2" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="H64" s="2">
         <v>2.0</v>
@@ -9506,16 +9512,16 @@
     </row>
     <row r="65" ht="15.75" customHeight="1">
       <c r="A65" s="2" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E65" s="2" t="s">
         <v>570</v>
@@ -9524,7 +9530,7 @@
         <v>580</v>
       </c>
       <c r="G65" s="2" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="H65" s="2">
         <v>3.0</v>
@@ -9541,16 +9547,16 @@
     </row>
     <row r="66" ht="15.75" customHeight="1">
       <c r="A66" s="2" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E66" s="2" t="s">
         <v>570</v>
@@ -9559,7 +9565,7 @@
         <v>580</v>
       </c>
       <c r="G66" s="2" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="H66" s="2">
         <v>4.0</v>
@@ -9576,16 +9582,16 @@
     </row>
     <row r="67" ht="15.75" customHeight="1">
       <c r="A67" s="2" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E67" s="2" t="s">
         <v>570</v>
@@ -9594,7 +9600,7 @@
         <v>580</v>
       </c>
       <c r="G67" s="2" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="H67" s="2">
         <v>1.0</v>
@@ -9611,16 +9617,16 @@
     </row>
     <row r="68" ht="15.75" customHeight="1">
       <c r="A68" s="2" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E68" s="2" t="s">
         <v>570</v>
@@ -9629,7 +9635,7 @@
         <v>580</v>
       </c>
       <c r="G68" s="2" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="H68" s="2">
         <v>2.0</v>
@@ -9646,16 +9652,16 @@
     </row>
     <row r="69" ht="15.75" customHeight="1">
       <c r="A69" s="2" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E69" s="2" t="s">
         <v>570</v>
@@ -9664,13 +9670,13 @@
         <v>580</v>
       </c>
       <c r="G69" s="2" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="H69" s="2">
         <v>3.0</v>
       </c>
       <c r="I69" s="2" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="J69" s="1" t="s">
         <v>291</v>
@@ -9681,16 +9687,16 @@
     </row>
     <row r="70" ht="15.75" customHeight="1">
       <c r="A70" s="2" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E70" s="2" t="s">
         <v>570</v>
@@ -9699,7 +9705,7 @@
         <v>580</v>
       </c>
       <c r="G70" s="2" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="H70" s="2">
         <v>4.0</v>
@@ -9716,16 +9722,16 @@
     </row>
     <row r="71" ht="15.75" customHeight="1">
       <c r="A71" s="2" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E71" s="2" t="s">
         <v>570</v>
@@ -9734,13 +9740,13 @@
         <v>580</v>
       </c>
       <c r="G71" s="2" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="H71" s="2">
         <v>1.0</v>
       </c>
       <c r="I71" s="2" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="J71" s="1" t="s">
         <v>169</v>
@@ -9751,16 +9757,16 @@
     </row>
     <row r="72" ht="15.75" customHeight="1">
       <c r="A72" s="2" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E72" s="2" t="s">
         <v>570</v>
@@ -9769,13 +9775,13 @@
         <v>580</v>
       </c>
       <c r="G72" s="2" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="H72" s="2">
         <v>2.0</v>
       </c>
       <c r="I72" s="2" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="J72" s="1" t="s">
         <v>220</v>
@@ -9786,16 +9792,16 @@
     </row>
     <row r="73" ht="15.75" customHeight="1">
       <c r="A73" s="2" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E73" s="2" t="s">
         <v>570</v>
@@ -9804,13 +9810,13 @@
         <v>580</v>
       </c>
       <c r="G73" s="2" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="H73" s="2">
         <v>3.0</v>
       </c>
       <c r="I73" s="2" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="J73" s="1" t="s">
         <v>244</v>
@@ -9821,16 +9827,16 @@
     </row>
     <row r="74" ht="15.75" customHeight="1">
       <c r="A74" s="2" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E74" s="2" t="s">
         <v>570</v>
@@ -9839,13 +9845,13 @@
         <v>580</v>
       </c>
       <c r="G74" s="2" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="H74" s="2">
         <v>4.0</v>
       </c>
       <c r="I74" s="2" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="J74" s="1" t="s">
         <v>211</v>
@@ -9856,16 +9862,16 @@
     </row>
     <row r="75" ht="15.75" customHeight="1">
       <c r="A75" s="2" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E75" s="2" t="s">
         <v>570</v>
@@ -9874,7 +9880,7 @@
         <v>580</v>
       </c>
       <c r="G75" s="2" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="H75" s="2">
         <v>5.0</v>
@@ -9891,16 +9897,16 @@
     </row>
     <row r="76" ht="15.75" customHeight="1">
       <c r="A76" s="2" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="E76" s="2" t="s">
         <v>570</v>
@@ -9909,7 +9915,7 @@
         <v>580</v>
       </c>
       <c r="G76" s="2" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="H76" s="2">
         <v>1.0</v>
@@ -9926,16 +9932,16 @@
     </row>
     <row r="77" ht="15.75" customHeight="1">
       <c r="A77" s="2" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="E77" s="2" t="s">
         <v>570</v>
@@ -9944,13 +9950,13 @@
         <v>580</v>
       </c>
       <c r="G77" s="2" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="H77" s="2">
         <v>2.0</v>
       </c>
       <c r="I77" s="2" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="J77" s="1" t="s">
         <v>199</v>
@@ -9961,16 +9967,16 @@
     </row>
     <row r="78" ht="15.75" customHeight="1">
       <c r="A78" s="2" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="E78" s="2" t="s">
         <v>570</v>
@@ -9979,13 +9985,13 @@
         <v>580</v>
       </c>
       <c r="G78" s="2" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="H78" s="2">
         <v>3.0</v>
       </c>
       <c r="I78" s="2" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="J78" s="2" t="s">
         <v>461</v>
@@ -9996,16 +10002,16 @@
     </row>
     <row r="79" ht="15.75" customHeight="1">
       <c r="A79" s="2" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="E79" s="2" t="s">
         <v>570</v>
@@ -10014,13 +10020,13 @@
         <v>580</v>
       </c>
       <c r="G79" s="2" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="H79" s="2">
         <v>4.0</v>
       </c>
       <c r="I79" s="2" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="J79" s="1" t="s">
         <v>178</v>
@@ -10031,16 +10037,16 @@
     </row>
     <row r="80" ht="15.75" customHeight="1">
       <c r="A80" s="2" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="E80" s="2" t="s">
         <v>570</v>
@@ -10049,13 +10055,13 @@
         <v>580</v>
       </c>
       <c r="G80" s="2" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="H80" s="2">
         <v>1.0</v>
       </c>
       <c r="I80" s="2" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="J80" s="1" t="s">
         <v>342</v>
@@ -10066,16 +10072,16 @@
     </row>
     <row r="81" ht="15.75" customHeight="1">
       <c r="A81" s="2" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="E81" s="2" t="s">
         <v>570</v>
@@ -10084,13 +10090,13 @@
         <v>580</v>
       </c>
       <c r="G81" s="2" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="H81" s="2">
         <v>2.0</v>
       </c>
       <c r="I81" s="2" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="J81" s="1" t="s">
         <v>172</v>
@@ -10101,16 +10107,16 @@
     </row>
     <row r="82" ht="15.75" customHeight="1">
       <c r="A82" s="2" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="E82" s="2" t="s">
         <v>570</v>
@@ -10119,13 +10125,13 @@
         <v>580</v>
       </c>
       <c r="G82" s="2" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="H82" s="2">
         <v>3.0</v>
       </c>
       <c r="I82" s="2" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="J82" s="1" t="s">
         <v>449</v>
@@ -10136,16 +10142,16 @@
     </row>
     <row r="83" ht="15.75" customHeight="1">
       <c r="A83" s="2" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="E83" s="2" t="s">
         <v>570</v>
@@ -10154,13 +10160,13 @@
         <v>580</v>
       </c>
       <c r="G83" s="2" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="H83" s="2">
         <v>4.0</v>
       </c>
       <c r="I83" s="2" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="J83" s="1" t="s">
         <v>339</v>
@@ -10171,16 +10177,16 @@
     </row>
     <row r="84" ht="15.75" customHeight="1">
       <c r="A84" s="2" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="E84" s="2" t="s">
         <v>570</v>
@@ -10189,7 +10195,7 @@
         <v>580</v>
       </c>
       <c r="G84" s="2" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="H84" s="2">
         <v>1.0</v>
@@ -10206,16 +10212,16 @@
     </row>
     <row r="85" ht="15.75" customHeight="1">
       <c r="A85" s="2" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="E85" s="2" t="s">
         <v>570</v>
@@ -10224,7 +10230,7 @@
         <v>580</v>
       </c>
       <c r="G85" s="2" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="H85" s="2">
         <v>2.0</v>
@@ -10241,16 +10247,16 @@
     </row>
     <row r="86" ht="15.75" customHeight="1">
       <c r="A86" s="2" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="E86" s="2" t="s">
         <v>570</v>
@@ -10259,13 +10265,13 @@
         <v>580</v>
       </c>
       <c r="G86" s="2" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="H86" s="2">
         <v>3.0</v>
       </c>
       <c r="I86" s="2" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="J86" s="1" t="s">
         <v>336</v>
@@ -10276,16 +10282,16 @@
     </row>
     <row r="87" ht="15.75" customHeight="1">
       <c r="A87" s="2" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="E87" s="2" t="s">
         <v>570</v>
@@ -10294,7 +10300,7 @@
         <v>580</v>
       </c>
       <c r="G87" s="2" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="H87" s="2">
         <v>4.0</v>
@@ -10311,16 +10317,16 @@
     </row>
     <row r="88" ht="15.75" customHeight="1">
       <c r="A88" s="2" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="E88" s="2" t="s">
         <v>570</v>
@@ -10329,7 +10335,7 @@
         <v>580</v>
       </c>
       <c r="G88" s="2" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="H88" s="2">
         <v>1.0</v>
@@ -10346,16 +10352,16 @@
     </row>
     <row r="89" ht="15.75" customHeight="1">
       <c r="A89" s="2" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="E89" s="2" t="s">
         <v>570</v>
@@ -10364,7 +10370,7 @@
         <v>580</v>
       </c>
       <c r="G89" s="2" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="H89" s="2">
         <v>2.0</v>
@@ -10381,16 +10387,16 @@
     </row>
     <row r="90" ht="15.75" customHeight="1">
       <c r="A90" s="2" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="E90" s="2" t="s">
         <v>570</v>
@@ -10399,7 +10405,7 @@
         <v>580</v>
       </c>
       <c r="G90" s="2" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="H90" s="2">
         <v>3.0</v>
@@ -10416,16 +10422,16 @@
     </row>
     <row r="91" ht="15.75" customHeight="1">
       <c r="A91" s="2" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="E91" s="2" t="s">
         <v>570</v>
@@ -10434,7 +10440,7 @@
         <v>580</v>
       </c>
       <c r="G91" s="2" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="H91" s="2">
         <v>4.0</v>
@@ -10451,16 +10457,16 @@
     </row>
     <row r="92" ht="15.75" customHeight="1">
       <c r="A92" s="2" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="E92" s="2" t="s">
         <v>570</v>
@@ -10469,7 +10475,7 @@
         <v>580</v>
       </c>
       <c r="G92" s="2" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="H92" s="2">
         <v>5.0</v>
@@ -10486,16 +10492,16 @@
     </row>
     <row r="93" ht="15.75" customHeight="1">
       <c r="A93" s="2" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="E93" s="2" t="s">
         <v>570</v>
@@ -10504,7 +10510,7 @@
         <v>580</v>
       </c>
       <c r="G93" s="2" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="H93" s="2">
         <v>6.0</v>
@@ -10521,16 +10527,16 @@
     </row>
     <row r="94" ht="15.75" customHeight="1">
       <c r="A94" s="2" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="E94" s="2" t="s">
         <v>570</v>
@@ -10539,7 +10545,7 @@
         <v>580</v>
       </c>
       <c r="G94" s="2" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="H94" s="2">
         <v>7.0</v>
@@ -10556,16 +10562,16 @@
     </row>
     <row r="95" ht="15.75" customHeight="1">
       <c r="A95" s="2" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="E95" s="2" t="s">
         <v>570</v>
@@ -10574,7 +10580,7 @@
         <v>580</v>
       </c>
       <c r="G95" s="2" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="H95" s="2">
         <v>8.0</v>
@@ -10591,16 +10597,16 @@
     </row>
     <row r="96" ht="15.75" customHeight="1">
       <c r="A96" s="2" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="E96" s="2" t="s">
         <v>588</v>
@@ -10609,13 +10615,13 @@
         <v>580</v>
       </c>
       <c r="G96" s="2" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="H96" s="2">
         <v>1.0</v>
       </c>
       <c r="I96" s="2" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="J96" s="1" t="s">
         <v>53</v>
@@ -10626,16 +10632,16 @@
     </row>
     <row r="97" ht="15.75" customHeight="1">
       <c r="A97" s="2" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="E97" s="2" t="s">
         <v>588</v>
@@ -10644,7 +10650,7 @@
         <v>580</v>
       </c>
       <c r="G97" s="2" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="H97" s="2">
         <v>2.0</v>
@@ -10661,16 +10667,16 @@
     </row>
     <row r="98" ht="15.75" customHeight="1">
       <c r="A98" s="2" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="E98" s="2" t="s">
         <v>588</v>
@@ -10679,13 +10685,13 @@
         <v>580</v>
       </c>
       <c r="G98" s="2" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="H98" s="2">
         <v>3.0</v>
       </c>
       <c r="I98" s="2" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="J98" s="1" t="s">
         <v>126</v>
@@ -10696,16 +10702,16 @@
     </row>
     <row r="99" ht="15.75" customHeight="1">
       <c r="A99" s="2" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="E99" s="2" t="s">
         <v>588</v>
@@ -10714,7 +10720,7 @@
         <v>580</v>
       </c>
       <c r="G99" s="2" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="H99" s="2">
         <v>4.0</v>
@@ -10731,16 +10737,16 @@
     </row>
     <row r="100" ht="15.75" customHeight="1">
       <c r="A100" s="2" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="E100" s="2" t="s">
         <v>588</v>
@@ -10749,13 +10755,13 @@
         <v>580</v>
       </c>
       <c r="G100" s="2" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="H100" s="2">
         <v>5.0</v>
       </c>
       <c r="I100" s="2" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="J100" s="1" t="s">
         <v>68</v>
@@ -10766,16 +10772,16 @@
     </row>
     <row r="101" ht="15.75" customHeight="1">
       <c r="A101" s="2" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="E101" s="2" t="s">
         <v>588</v>
@@ -10784,7 +10790,7 @@
         <v>580</v>
       </c>
       <c r="G101" s="2" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="H101" s="2">
         <v>1.0</v>
@@ -10801,16 +10807,16 @@
     </row>
     <row r="102" ht="15.75" customHeight="1">
       <c r="A102" s="2" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="D102" s="2" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="E102" s="2" t="s">
         <v>588</v>
@@ -10819,13 +10825,13 @@
         <v>580</v>
       </c>
       <c r="G102" s="2" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="H102" s="2">
         <v>2.0</v>
       </c>
       <c r="I102" s="2" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="J102" s="1" t="s">
         <v>309</v>
@@ -10836,16 +10842,16 @@
     </row>
     <row r="103" ht="15.75" customHeight="1">
       <c r="A103" s="2" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="D103" s="2" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="E103" s="2" t="s">
         <v>588</v>
@@ -10854,13 +10860,13 @@
         <v>580</v>
       </c>
       <c r="G103" s="2" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="H103" s="2">
         <v>3.0</v>
       </c>
-      <c r="I103" s="1" t="s">
-        <v>208</v>
+      <c r="I103" s="2" t="s">
+        <v>696</v>
       </c>
       <c r="J103" s="1" t="s">
         <v>208</v>
@@ -10871,16 +10877,16 @@
     </row>
     <row r="104" ht="15.75" customHeight="1">
       <c r="A104" s="2" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="D104" s="2" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="E104" s="2" t="s">
         <v>588</v>
@@ -10889,13 +10895,13 @@
         <v>580</v>
       </c>
       <c r="G104" s="2" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="H104" s="2">
         <v>4.0</v>
       </c>
       <c r="I104" s="2" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
       <c r="J104" s="1" t="s">
         <v>62</v>
@@ -10906,16 +10912,16 @@
     </row>
     <row r="105" ht="15.75" customHeight="1">
       <c r="A105" s="2" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="D105" s="2" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="E105" s="2" t="s">
         <v>588</v>
@@ -10924,7 +10930,7 @@
         <v>580</v>
       </c>
       <c r="G105" s="2" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="H105" s="2">
         <v>5.0</v>
@@ -10941,16 +10947,16 @@
     </row>
     <row r="106" ht="15.75" customHeight="1">
       <c r="A106" s="2" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="C106" s="2" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="D106" s="2" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="E106" s="2" t="s">
         <v>588</v>
@@ -10959,7 +10965,7 @@
         <v>580</v>
       </c>
       <c r="G106" s="2" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="H106" s="2">
         <v>6.0</v>
@@ -10976,16 +10982,16 @@
     </row>
     <row r="107" ht="15.75" customHeight="1">
       <c r="A107" s="2" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="D107" s="2" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="E107" s="2" t="s">
         <v>588</v>
@@ -10994,13 +11000,13 @@
         <v>580</v>
       </c>
       <c r="G107" s="2" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="H107" s="2">
         <v>7.0</v>
       </c>
       <c r="I107" s="2" t="s">
-        <v>696</v>
+        <v>698</v>
       </c>
       <c r="J107" s="1" t="s">
         <v>440</v>
@@ -11011,16 +11017,16 @@
     </row>
     <row r="108" ht="15.75" customHeight="1">
       <c r="A108" s="2" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="D108" s="2" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="E108" s="2" t="s">
         <v>588</v>
@@ -11029,13 +11035,13 @@
         <v>580</v>
       </c>
       <c r="G108" s="2" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="H108" s="2">
         <v>8.0</v>
       </c>
       <c r="I108" s="2" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
       <c r="J108" s="1" t="s">
         <v>65</v>
@@ -11046,16 +11052,16 @@
     </row>
     <row r="109" ht="15.75" customHeight="1">
       <c r="A109" s="2" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
       <c r="D109" s="2" t="s">
-        <v>701</v>
+        <v>703</v>
       </c>
       <c r="E109" s="2" t="s">
         <v>588</v>
@@ -11064,13 +11070,13 @@
         <v>580</v>
       </c>
       <c r="G109" s="2" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="H109" s="2">
         <v>1.0</v>
       </c>
       <c r="I109" s="2" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
       <c r="J109" s="1" t="s">
         <v>184</v>
@@ -11081,16 +11087,16 @@
     </row>
     <row r="110" ht="15.75" customHeight="1">
       <c r="A110" s="2" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
       <c r="D110" s="2" t="s">
-        <v>701</v>
+        <v>703</v>
       </c>
       <c r="E110" s="2" t="s">
         <v>588</v>
@@ -11099,13 +11105,13 @@
         <v>580</v>
       </c>
       <c r="G110" s="2" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="H110" s="2">
         <v>2.0</v>
       </c>
       <c r="I110" s="2" t="s">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="J110" s="1" t="s">
         <v>300</v>
@@ -11116,16 +11122,16 @@
     </row>
     <row r="111" ht="15.75" customHeight="1">
       <c r="A111" s="2" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
       <c r="D111" s="2" t="s">
-        <v>701</v>
+        <v>703</v>
       </c>
       <c r="E111" s="2" t="s">
         <v>588</v>
@@ -11134,7 +11140,7 @@
         <v>580</v>
       </c>
       <c r="G111" s="2" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="H111" s="2">
         <v>3.0</v>
@@ -11151,16 +11157,16 @@
     </row>
     <row r="112" ht="15.75" customHeight="1">
       <c r="A112" s="2" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
       <c r="C112" s="2" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
       <c r="D112" s="2" t="s">
-        <v>701</v>
+        <v>703</v>
       </c>
       <c r="E112" s="2" t="s">
         <v>588</v>
@@ -11169,13 +11175,13 @@
         <v>580</v>
       </c>
       <c r="G112" s="2" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="H112" s="2">
         <v>4.0</v>
       </c>
       <c r="I112" s="2" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
       <c r="J112" s="1" t="s">
         <v>91</v>
@@ -11186,16 +11192,16 @@
     </row>
     <row r="113" ht="15.75" customHeight="1">
       <c r="A113" s="2" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
       <c r="D113" s="2" t="s">
-        <v>701</v>
+        <v>703</v>
       </c>
       <c r="E113" s="2" t="s">
         <v>588</v>
@@ -11204,13 +11210,13 @@
         <v>580</v>
       </c>
       <c r="G113" s="2" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="H113" s="2">
         <v>5.0</v>
       </c>
       <c r="I113" s="2" t="s">
-        <v>706</v>
+        <v>708</v>
       </c>
       <c r="J113" s="1" t="s">
         <v>202</v>
@@ -11221,16 +11227,16 @@
     </row>
     <row r="114" ht="15.75" customHeight="1">
       <c r="A114" s="2" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>709</v>
+        <v>711</v>
       </c>
       <c r="D114" s="2" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="E114" s="2" t="s">
         <v>553</v>
@@ -11239,13 +11245,13 @@
         <v>580</v>
       </c>
       <c r="G114" s="2" t="s">
-        <v>711</v>
+        <v>713</v>
       </c>
       <c r="H114" s="2">
         <v>1.0</v>
       </c>
       <c r="I114" s="2" t="s">
-        <v>712</v>
+        <v>714</v>
       </c>
       <c r="J114" s="1" t="s">
         <v>104</v>
@@ -11256,16 +11262,16 @@
     </row>
     <row r="115" ht="15.75" customHeight="1">
       <c r="A115" s="2" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>709</v>
+        <v>711</v>
       </c>
       <c r="D115" s="2" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="E115" s="2" t="s">
         <v>553</v>
@@ -11274,13 +11280,13 @@
         <v>580</v>
       </c>
       <c r="G115" s="2" t="s">
-        <v>711</v>
+        <v>713</v>
       </c>
       <c r="H115" s="2">
         <v>2.0</v>
       </c>
       <c r="I115" s="2" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
       <c r="J115" s="2" t="s">
         <v>360</v>

</xml_diff>

<commit_message>
Refresh shrine and course data from workbook
</commit_message>
<xml_diff>
--- a/korean_catholic_holy_sites.xlsx
+++ b/korean_catholic_holy_sites.xlsx
@@ -10690,11 +10690,11 @@
       <c r="H98" s="2">
         <v>3.0</v>
       </c>
-      <c r="I98" s="2" t="s">
-        <v>690</v>
+      <c r="I98" s="1" t="s">
+        <v>17</v>
       </c>
       <c r="J98" s="1" t="s">
-        <v>126</v>
+        <v>17</v>
       </c>
       <c r="K98" s="5" t="s">
         <v>557</v>
@@ -10725,11 +10725,11 @@
       <c r="H99" s="2">
         <v>4.0</v>
       </c>
-      <c r="I99" s="1" t="s">
-        <v>17</v>
+      <c r="I99" s="2" t="s">
+        <v>690</v>
       </c>
       <c r="J99" s="1" t="s">
-        <v>17</v>
+        <v>126</v>
       </c>
       <c r="K99" s="5" t="s">
         <v>557</v>

</xml_diff>

<commit_message>
Update workbook address and geocoded data
</commit_message>
<xml_diff>
--- a/korean_catholic_holy_sites.xlsx
+++ b/korean_catholic_holy_sites.xlsx
@@ -1100,7 +1100,7 @@
     <t>용수 성지</t>
   </si>
   <si>
-    <t>제주특별자치도 제주시 한경면 용수1길 108</t>
+    <t>제주특별자치도 한경면 용수1길 108</t>
   </si>
   <si>
     <t>128</t>
@@ -4416,7 +4416,7 @@
       <c r="D114" s="2" t="s">
         <v>360</v>
       </c>
-      <c r="E114" s="1" t="s">
+      <c r="E114" s="2" t="s">
         <v>361</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Refine course detail panel and workbook
</commit_message>
<xml_diff>
--- a/korean_catholic_holy_sites.xlsx
+++ b/korean_catholic_holy_sites.xlsx
@@ -1697,13 +1697,13 @@
     <t>의금부-터</t>
   </si>
   <si>
+    <t>우포도청-터</t>
+  </si>
+  <si>
+    <t>전옥서-터</t>
+  </si>
+  <si>
     <t>좌포도청-터</t>
-  </si>
-  <si>
-    <t>전옥서-터</t>
-  </si>
-  <si>
-    <t>우포도청-터</t>
   </si>
   <si>
     <t>seoul2_course</t>
@@ -7439,7 +7439,7 @@
         <v>560</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>419</v>
+        <v>366</v>
       </c>
       <c r="K5" s="5" t="s">
         <v>557</v>
@@ -7509,7 +7509,7 @@
         <v>562</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>366</v>
+        <v>419</v>
       </c>
       <c r="K7" s="5" t="s">
         <v>557</v>

</xml_diff>